<commit_message>
Regenerate ddPCR results from raw workflow
</commit_message>
<xml_diff>
--- a/results/ddPCR/SNV_pooled_participant.xlsx
+++ b/results/ddPCR/SNV_pooled_participant.xlsx
@@ -737,22 +737,22 @@
         <v>91831</v>
       </c>
       <c r="I2" t="n">
-        <v>0.00129585869695419</v>
+        <v>0.0274386402820978</v>
       </c>
       <c r="J2" t="n">
-        <v>0.00107362503182806</v>
+        <v>0.022719714304557</v>
       </c>
       <c r="K2" t="n">
-        <v>0.00155049050629918</v>
+        <v>0.0328535400849928</v>
       </c>
       <c r="L2" t="n">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="M2" t="n">
-        <v>0.000762269821737757</v>
+        <v>0.141564395465584</v>
       </c>
       <c r="N2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="b">
         <v>0</v>
@@ -784,22 +784,22 @@
         <v>87610</v>
       </c>
       <c r="I3" t="n">
-        <v>0.00131263554388768</v>
+        <v>0.0253201539099395</v>
       </c>
       <c r="J3" t="n">
-        <v>0.00108383316937011</v>
+        <v>0.0208902241817673</v>
       </c>
       <c r="K3" t="n">
-        <v>0.00157541294615648</v>
+        <v>0.0304178244175161</v>
       </c>
       <c r="L3" t="n">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="M3" t="n">
-        <v>0.000821823992694898</v>
+        <v>0.151809154206141</v>
       </c>
       <c r="N3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" t="b">
         <v>0</v>
@@ -831,22 +831,22 @@
         <v>78867</v>
       </c>
       <c r="I4" t="n">
-        <v>0.00167370383049945</v>
+        <v>0.0405321252882686</v>
       </c>
       <c r="J4" t="n">
-        <v>0.00140055675219997</v>
+        <v>0.0338993314657685</v>
       </c>
       <c r="K4" t="n">
-        <v>0.00198449037414683</v>
+        <v>0.0480890772302299</v>
       </c>
       <c r="L4" t="n">
-        <v>79</v>
+        <v>152</v>
       </c>
       <c r="M4" t="n">
-        <v>0.00100168638340497</v>
+        <v>0.192729531996906</v>
       </c>
       <c r="N4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" t="b">
         <v>0</v>
@@ -878,22 +878,22 @@
         <v>82870</v>
       </c>
       <c r="I5" t="n">
-        <v>0.00130324604802703</v>
+        <v>0.0291683799986658</v>
       </c>
       <c r="J5" t="n">
-        <v>0.00106919676350592</v>
+        <v>0.0239172140132913</v>
       </c>
       <c r="K5" t="n">
-        <v>0.00157324833205752</v>
+        <v>0.0352345376694111</v>
       </c>
       <c r="L5" t="n">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="M5" t="n">
-        <v>0.000760226861349101</v>
+        <v>0.14239169783999</v>
       </c>
       <c r="N5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" t="b">
         <v>0</v>
@@ -925,22 +925,22 @@
         <v>83753</v>
       </c>
       <c r="I6" t="n">
-        <v>0.00121786682268098</v>
+        <v>0.0279045939839292</v>
       </c>
       <c r="J6" t="n">
-        <v>0.000993130598311853</v>
+        <v>0.0227442223249464</v>
       </c>
       <c r="K6" t="n">
-        <v>0.00147821459595543</v>
+        <v>0.0338902090542832</v>
       </c>
       <c r="L6" t="n">
-        <v>69</v>
+        <v>127</v>
       </c>
       <c r="M6" t="n">
-        <v>0.00082385108593125</v>
+        <v>0.151636359294592</v>
       </c>
       <c r="N6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" t="b">
         <v>0</v>
@@ -972,22 +972,22 @@
         <v>87067</v>
       </c>
       <c r="I7" t="n">
-        <v>0.00142419056588604</v>
+        <v>0.0412889341683018</v>
       </c>
       <c r="J7" t="n">
-        <v>0.00118470320981456</v>
+        <v>0.0343344112870499</v>
       </c>
       <c r="K7" t="n">
-        <v>0.00169781966165938</v>
+        <v>0.0492418304374687</v>
       </c>
       <c r="L7" t="n">
-        <v>86</v>
+        <v>167</v>
       </c>
       <c r="M7" t="n">
-        <v>0.000987745069888706</v>
+        <v>0.191806310083039</v>
       </c>
       <c r="N7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" t="b">
         <v>0</v>
@@ -1019,22 +1019,22 @@
         <v>90502</v>
       </c>
       <c r="I8" t="n">
-        <v>0.00201100528165123</v>
+        <v>0.0296889080532411</v>
       </c>
       <c r="J8" t="n">
-        <v>0.00172967816922287</v>
+        <v>0.0254637579093407</v>
       </c>
       <c r="K8" t="n">
-        <v>0.00232497508526486</v>
+        <v>0.0344300967018523</v>
       </c>
       <c r="L8" t="n">
-        <v>135</v>
+        <v>256</v>
       </c>
       <c r="M8" t="n">
-        <v>0.00149167974188416</v>
+        <v>0.282866676979514</v>
       </c>
       <c r="N8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" t="b">
         <v>0</v>
@@ -1066,22 +1066,22 @@
         <v>91460</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0017603323857424</v>
+        <v>0.0269604404879219</v>
       </c>
       <c r="J9" t="n">
-        <v>0.00149910658282726</v>
+        <v>0.0229094737504563</v>
       </c>
       <c r="K9" t="n">
-        <v>0.00205392400160809</v>
+        <v>0.0315340655634852</v>
       </c>
       <c r="L9" t="n">
-        <v>87</v>
+        <v>166</v>
       </c>
       <c r="M9" t="n">
-        <v>0.000951235512792478</v>
+        <v>0.181500109337415</v>
       </c>
       <c r="N9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" t="b">
         <v>0</v>
@@ -1113,22 +1113,22 @@
         <v>95848</v>
       </c>
       <c r="I10" t="n">
-        <v>0.00127284867707203</v>
+        <v>0.0220558582329469</v>
       </c>
       <c r="J10" t="n">
-        <v>0.00105713249055839</v>
+        <v>0.0182983942994186</v>
       </c>
       <c r="K10" t="n">
-        <v>0.00151959540653146</v>
+        <v>0.0263647845229687</v>
       </c>
       <c r="L10" t="n">
-        <v>94</v>
+        <v>183</v>
       </c>
       <c r="M10" t="n">
-        <v>0.000980719472498122</v>
+        <v>0.190927301560805</v>
       </c>
       <c r="N10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O10" t="b">
         <v>0</v>
@@ -1160,22 +1160,22 @@
         <v>88163</v>
       </c>
       <c r="I11" t="n">
-        <v>0.00140648571396164</v>
+        <v>0.042454474102846</v>
       </c>
       <c r="J11" t="n">
-        <v>0.00116997388913631</v>
+        <v>0.0353044246084021</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0016767160404989</v>
+        <v>0.0506305083673122</v>
       </c>
       <c r="L11" t="n">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="M11" t="n">
-        <v>0.000759955990608305</v>
+        <v>0.141782834068714</v>
       </c>
       <c r="N11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11" t="b">
         <v>0</v>
@@ -1207,22 +1207,22 @@
         <v>88866</v>
       </c>
       <c r="I12" t="n">
-        <v>0.00119280714784057</v>
+        <v>0.0333228963656859</v>
       </c>
       <c r="J12" t="n">
-        <v>0.000976672885791396</v>
+        <v>0.0272761607573691</v>
       </c>
       <c r="K12" t="n">
-        <v>0.00144248561642246</v>
+        <v>0.0403139459986585</v>
       </c>
       <c r="L12" t="n">
-        <v>73</v>
+        <v>135</v>
       </c>
       <c r="M12" t="n">
-        <v>0.000821461526343033</v>
+        <v>0.151914117885355</v>
       </c>
       <c r="N12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O12" t="b">
         <v>0</v>
@@ -1254,22 +1254,22 @@
         <v>87822</v>
       </c>
       <c r="I13" t="n">
-        <v>0.00127530687071577</v>
+        <v>0.0430429256534968</v>
       </c>
       <c r="J13" t="n">
-        <v>0.00105019605010381</v>
+        <v>0.0354362341981335</v>
       </c>
       <c r="K13" t="n">
-        <v>0.001534326621764</v>
+        <v>0.0518012977776883</v>
       </c>
       <c r="L13" t="n">
-        <v>87</v>
+        <v>169</v>
       </c>
       <c r="M13" t="n">
-        <v>0.000990640158502425</v>
+        <v>0.192434697456218</v>
       </c>
       <c r="N13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O13" t="b">
         <v>0</v>
@@ -1301,19 +1301,19 @@
         <v>68031</v>
       </c>
       <c r="I14" t="n">
-        <v>0.000191089356322853</v>
+        <v>0.0126585875672502</v>
       </c>
       <c r="J14" t="n">
-        <v>0.000101750831950964</v>
+        <v>0.00674017519725735</v>
       </c>
       <c r="K14" t="n">
-        <v>0.000326746451142168</v>
+        <v>0.0216468968986501</v>
       </c>
       <c r="L14" t="n">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="M14" t="n">
-        <v>0.000367479531390102</v>
+        <v>0.101424350663668</v>
       </c>
       <c r="N14" t="b">
         <v>0</v>
@@ -1348,19 +1348,19 @@
         <v>65945</v>
       </c>
       <c r="I15" t="n">
-        <v>0.000394267950564865</v>
+        <v>0.0259927395763175</v>
       </c>
       <c r="J15" t="n">
-        <v>0.000257564570647184</v>
+        <v>0.0169792656392651</v>
       </c>
       <c r="K15" t="n">
-        <v>0.000577640913968613</v>
+        <v>0.0380861710614925</v>
       </c>
       <c r="L15" t="n">
-        <v>45</v>
+        <v>88</v>
       </c>
       <c r="M15" t="n">
-        <v>0.000682386837516112</v>
+        <v>0.133444537114262</v>
       </c>
       <c r="N15" t="b">
         <v>0</v>
@@ -1395,19 +1395,19 @@
         <v>73435</v>
       </c>
       <c r="I16" t="n">
-        <v>0.000558316878872472</v>
+        <v>0.0230210107144229</v>
       </c>
       <c r="J16" t="n">
-        <v>0.000400686692921037</v>
+        <v>0.0165192859927447</v>
       </c>
       <c r="K16" t="n">
-        <v>0.000757344481899569</v>
+        <v>0.031233474559758</v>
       </c>
       <c r="L16" t="n">
-        <v>55</v>
+        <v>111</v>
       </c>
       <c r="M16" t="n">
-        <v>0.000748961666780146</v>
+        <v>0.151154081841084</v>
       </c>
       <c r="N16" t="b">
         <v>0</v>
@@ -1442,19 +1442,19 @@
         <v>84651</v>
       </c>
       <c r="I17" t="n">
-        <v>0.00118132095308974</v>
+        <v>0.030283139964908</v>
       </c>
       <c r="J17" t="n">
-        <v>0.000961270038314255</v>
+        <v>0.0246328570103583</v>
       </c>
       <c r="K17" t="n">
-        <v>0.00143661922419847</v>
+        <v>0.0368449595471133</v>
       </c>
       <c r="L17" t="n">
-        <v>121</v>
+        <v>200</v>
       </c>
       <c r="M17" t="n">
-        <v>0.00142939835323859</v>
+        <v>0.236264190617949</v>
       </c>
       <c r="N17" t="b">
         <v>0</v>
@@ -1489,22 +1489,22 @@
         <v>90821</v>
       </c>
       <c r="I18" t="n">
-        <v>0.00190484579557591</v>
+        <v>0.0514092045052246</v>
       </c>
       <c r="J18" t="n">
-        <v>0.00163178074151815</v>
+        <v>0.044020382359506</v>
       </c>
       <c r="K18" t="n">
-        <v>0.00221046577949158</v>
+        <v>0.0596879993344228</v>
       </c>
       <c r="L18" t="n">
-        <v>168</v>
+        <v>334</v>
       </c>
       <c r="M18" t="n">
-        <v>0.00184979244888297</v>
+        <v>0.367756355908876</v>
       </c>
       <c r="N18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O18" t="b">
         <v>0</v>
@@ -1536,19 +1536,19 @@
         <v>75758</v>
       </c>
       <c r="I19" t="n">
-        <v>0.000329998152010349</v>
+        <v>0.0183859993876189</v>
       </c>
       <c r="J19" t="n">
-        <v>0.00021356842971787</v>
+        <v>0.0118982713278667</v>
       </c>
       <c r="K19" t="n">
-        <v>0.000487104093630397</v>
+        <v>0.0271423035055794</v>
       </c>
       <c r="L19" t="n">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="M19" t="n">
-        <v>0.000369597930251591</v>
+        <v>0.101639430819187</v>
       </c>
       <c r="N19" t="b">
         <v>0</v>
@@ -1583,19 +1583,19 @@
         <v>82536</v>
       </c>
       <c r="I20" t="n">
-        <v>0.000496752932053892</v>
+        <v>0.0301552624781032</v>
       </c>
       <c r="J20" t="n">
-        <v>0.000356501327320347</v>
+        <v>0.0216396513389308</v>
       </c>
       <c r="K20" t="n">
-        <v>0.000673841749932902</v>
+        <v>0.0409102047461458</v>
       </c>
       <c r="L20" t="n">
-        <v>56</v>
+        <v>108</v>
       </c>
       <c r="M20" t="n">
-        <v>0.000678491809634584</v>
+        <v>0.130851991858098</v>
       </c>
       <c r="N20" t="b">
         <v>0</v>
@@ -1630,19 +1630,19 @@
         <v>114080</v>
       </c>
       <c r="I21" t="n">
-        <v>0.000411991584852735</v>
+        <v>0.0336842225837829</v>
       </c>
       <c r="J21" t="n">
-        <v>0.000302731135222278</v>
+        <v>0.0247501377177717</v>
       </c>
       <c r="K21" t="n">
-        <v>0.000547824247703721</v>
+        <v>0.0447927629386641</v>
       </c>
       <c r="L21" t="n">
-        <v>97</v>
+        <v>381</v>
       </c>
       <c r="M21" t="n">
-        <v>0.000850280504908836</v>
+        <v>0.333976157082749</v>
       </c>
       <c r="N21" t="b">
         <v>0</v>
@@ -1677,19 +1677,19 @@
         <v>81739</v>
       </c>
       <c r="I22" t="n">
-        <v>0.000966490903974847</v>
+        <v>0.0429458817384176</v>
       </c>
       <c r="J22" t="n">
-        <v>0.00076525231182023</v>
+        <v>0.033998340454641</v>
       </c>
       <c r="K22" t="n">
-        <v>0.00120439264838401</v>
+        <v>0.0535283755484627</v>
       </c>
       <c r="L22" t="n">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="M22" t="n">
-        <v>0.00143138526284882</v>
+        <v>0.237340804267241</v>
       </c>
       <c r="N22" t="b">
         <v>0</v>
@@ -1724,22 +1724,22 @@
         <v>90154</v>
       </c>
       <c r="I23" t="n">
-        <v>0.000965015418062427</v>
+        <v>0.0418049338415665</v>
       </c>
       <c r="J23" t="n">
-        <v>0.000773007757036592</v>
+        <v>0.0334817031091647</v>
       </c>
       <c r="K23" t="n">
-        <v>0.00119020882322285</v>
+        <v>0.0515710491993853</v>
       </c>
       <c r="L23" t="n">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="M23" t="n">
-        <v>0.000920646893094039</v>
+        <v>0.171928034252501</v>
       </c>
       <c r="N23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O23" t="b">
         <v>0</v>
@@ -1771,19 +1771,19 @@
         <v>85829</v>
       </c>
       <c r="I24" t="n">
-        <v>0.000943736965361358</v>
+        <v>0.0485968305211817</v>
       </c>
       <c r="J24" t="n">
-        <v>0.000749531830026573</v>
+        <v>0.0385912035461668</v>
       </c>
       <c r="K24" t="n">
-        <v>0.00117284441035814</v>
+        <v>0.0604052258265511</v>
       </c>
       <c r="L24" t="n">
-        <v>159</v>
+        <v>316</v>
       </c>
       <c r="M24" t="n">
-        <v>0.00185252070978341</v>
+        <v>0.368173927227394</v>
       </c>
       <c r="N24" t="b">
         <v>0</v>
@@ -1818,19 +1818,19 @@
         <v>70136</v>
       </c>
       <c r="I25" t="n">
-        <v>0.00106935097524809</v>
+        <v>0.0528260527467124</v>
       </c>
       <c r="J25" t="n">
-        <v>0.000841202399488483</v>
+        <v>0.0415486276459986</v>
       </c>
       <c r="K25" t="n">
-        <v>0.00134025898699808</v>
+        <v>0.0662233964706642</v>
       </c>
       <c r="L25" t="n">
-        <v>102</v>
+        <v>168</v>
       </c>
       <c r="M25" t="n">
-        <v>0.0014543173263374</v>
+        <v>0.239534618455572</v>
       </c>
       <c r="N25" t="b">
         <v>0</v>
@@ -1865,25 +1865,25 @@
         <v>181499</v>
       </c>
       <c r="I26" t="n">
-        <v>0.00269422972027394</v>
+        <v>0.125606358120142</v>
       </c>
       <c r="J26" t="n">
-        <v>0.00246097436752768</v>
+        <v>0.114709868958417</v>
       </c>
       <c r="K26" t="n">
-        <v>0.00294358726407673</v>
+        <v>0.137260692967258</v>
       </c>
       <c r="L26" t="n">
-        <v>158</v>
+        <v>300</v>
       </c>
       <c r="M26" t="n">
-        <v>0.000870528212276652</v>
+        <v>0.165290166887972</v>
       </c>
       <c r="N26" t="b">
         <v>1</v>
       </c>
       <c r="O26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1912,19 +1912,19 @@
         <v>77491</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0014195196861571</v>
+        <v>0.0676246715873225</v>
       </c>
       <c r="J27" t="n">
-        <v>0.00116681257314999</v>
+        <v>0.0555751503507957</v>
       </c>
       <c r="K27" t="n">
-        <v>0.00171065577092511</v>
+        <v>0.08151393479893</v>
       </c>
       <c r="L27" t="n">
-        <v>145</v>
+        <v>287</v>
       </c>
       <c r="M27" t="n">
-        <v>0.00187118504084345</v>
+        <v>0.370365590842808</v>
       </c>
       <c r="N27" t="b">
         <v>0</v>
@@ -1959,19 +1959,19 @@
         <v>78322</v>
       </c>
       <c r="I28" t="n">
-        <v>0.00125124486095861</v>
+        <v>0.0260215932002233</v>
       </c>
       <c r="J28" t="n">
-        <v>0.00101593419426638</v>
+        <v>0.0211142722873273</v>
       </c>
       <c r="K28" t="n">
-        <v>0.00152465804520896</v>
+        <v>0.0317329678233123</v>
       </c>
       <c r="L28" t="n">
-        <v>113</v>
+        <v>186</v>
       </c>
       <c r="M28" t="n">
-        <v>0.0014427619315135</v>
+        <v>0.237481167488062</v>
       </c>
       <c r="N28" t="b">
         <v>0</v>
@@ -2006,19 +2006,19 @@
         <v>94780</v>
       </c>
       <c r="I29" t="n">
-        <v>0.00184638109305761</v>
+        <v>0.0397445286632307</v>
       </c>
       <c r="J29" t="n">
-        <v>0.00158314878135979</v>
+        <v>0.0340552588161853</v>
       </c>
       <c r="K29" t="n">
-        <v>0.00214080777632009</v>
+        <v>0.0461185365203327</v>
       </c>
       <c r="L29" t="n">
-        <v>87</v>
+        <v>162</v>
       </c>
       <c r="M29" t="n">
-        <v>0.00091791517197721</v>
+        <v>0.170922135471618</v>
       </c>
       <c r="N29" t="b">
         <v>1</v>
@@ -2053,22 +2053,22 @@
         <v>89221</v>
       </c>
       <c r="I30" t="n">
-        <v>0.00210712724582778</v>
+        <v>0.0505261205414791</v>
       </c>
       <c r="J30" t="n">
-        <v>0.00181692976955916</v>
+        <v>0.0435422136848823</v>
       </c>
       <c r="K30" t="n">
-        <v>0.00243041696906221</v>
+        <v>0.0583176125606386</v>
       </c>
       <c r="L30" t="n">
-        <v>165</v>
+        <v>328</v>
       </c>
       <c r="M30" t="n">
-        <v>0.00184934040192331</v>
+        <v>0.367626455655059</v>
       </c>
       <c r="N30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O30" t="b">
         <v>0</v>
@@ -2100,19 +2100,19 @@
         <v>91262</v>
       </c>
       <c r="I31" t="n">
-        <v>0.000635532861431921</v>
+        <v>0.0231911357245898</v>
       </c>
       <c r="J31" t="n">
-        <v>0.000482621014901374</v>
+        <v>0.0176085998339115</v>
       </c>
       <c r="K31" t="n">
-        <v>0.000821497168474572</v>
+        <v>0.029983258387406</v>
       </c>
       <c r="L31" t="n">
-        <v>88</v>
+        <v>139</v>
       </c>
       <c r="M31" t="n">
-        <v>0.000964256755276019</v>
+        <v>0.152308737481098</v>
       </c>
       <c r="N31" t="b">
         <v>0</v>
@@ -2147,19 +2147,19 @@
         <v>91832</v>
       </c>
       <c r="I32" t="n">
-        <v>0.000664256468333479</v>
+        <v>0.0229563309349425</v>
       </c>
       <c r="J32" t="n">
-        <v>0.000508140477339381</v>
+        <v>0.017558155595385</v>
       </c>
       <c r="K32" t="n">
-        <v>0.000853184577426558</v>
+        <v>0.0294921094759439</v>
       </c>
       <c r="L32" t="n">
-        <v>88</v>
+        <v>166</v>
       </c>
       <c r="M32" t="n">
-        <v>0.000958271626448297</v>
+        <v>0.180764874989111</v>
       </c>
       <c r="N32" t="b">
         <v>0</v>
@@ -2194,19 +2194,19 @@
         <v>85905</v>
       </c>
       <c r="I33" t="n">
-        <v>0.000803212851405623</v>
+        <v>0.0361733552983198</v>
       </c>
       <c r="J33" t="n">
-        <v>0.000624999621030242</v>
+        <v>0.0281434089962867</v>
       </c>
       <c r="K33" t="n">
-        <v>0.00101640884309462</v>
+        <v>0.0457834108070701</v>
       </c>
       <c r="L33" t="n">
-        <v>85</v>
+        <v>160</v>
       </c>
       <c r="M33" t="n">
-        <v>0.000989465106804028</v>
+        <v>0.186252255398405</v>
       </c>
       <c r="N33" t="b">
         <v>0</v>
@@ -2241,19 +2241,19 @@
         <v>91571</v>
       </c>
       <c r="I34" t="n">
-        <v>0.000764434154918042</v>
+        <v>0.0170932050110588</v>
       </c>
       <c r="J34" t="n">
-        <v>0.000595960895559133</v>
+        <v>0.0133210112623035</v>
       </c>
       <c r="K34" t="n">
-        <v>0.000965719306105228</v>
+        <v>0.0216046657224494</v>
       </c>
       <c r="L34" t="n">
-        <v>88</v>
+        <v>139</v>
       </c>
       <c r="M34" t="n">
-        <v>0.000961002937611252</v>
+        <v>0.151794782190868</v>
       </c>
       <c r="N34" t="b">
         <v>0</v>
@@ -2288,19 +2288,19 @@
         <v>91934</v>
       </c>
       <c r="I35" t="n">
-        <v>0.000630887375726064</v>
+        <v>0.0135531654762694</v>
       </c>
       <c r="J35" t="n">
-        <v>0.00047909300364668</v>
+        <v>0.0102883957633695</v>
       </c>
       <c r="K35" t="n">
-        <v>0.000815492914258642</v>
+        <v>0.0175276818894564</v>
       </c>
       <c r="L35" t="n">
-        <v>79</v>
+        <v>145</v>
       </c>
       <c r="M35" t="n">
-        <v>0.000859312115213088</v>
+        <v>0.157721843931516</v>
       </c>
       <c r="N35" t="b">
         <v>0</v>
@@ -2335,19 +2335,19 @@
         <v>99167</v>
       </c>
       <c r="I36" t="n">
-        <v>0.000978147972611857</v>
+        <v>0.0210403743223182</v>
       </c>
       <c r="J36" t="n">
-        <v>0.000793281481428321</v>
+        <v>0.0170559128515269</v>
       </c>
       <c r="K36" t="n">
-        <v>0.0011931292131302</v>
+        <v>0.0256794891378054</v>
       </c>
       <c r="L36" t="n">
-        <v>97</v>
+        <v>333</v>
       </c>
       <c r="M36" t="n">
-        <v>0.000978147972611857</v>
+        <v>0.335797190597679</v>
       </c>
       <c r="N36" t="b">
         <v>0</v>
@@ -2382,22 +2382,22 @@
         <v>132006</v>
       </c>
       <c r="I37" t="n">
-        <v>0.00069693801796888</v>
+        <v>0.0149545398999578</v>
       </c>
       <c r="J37" t="n">
-        <v>0.000561866241130859</v>
+        <v>0.0120521585822811</v>
       </c>
       <c r="K37" t="n">
-        <v>0.00085466516672994</v>
+        <v>0.0183467624469577</v>
       </c>
       <c r="L37" t="n">
-        <v>82</v>
+        <v>366</v>
       </c>
       <c r="M37" t="n">
-        <v>0.000621183885580958</v>
+        <v>0.277260124539794</v>
       </c>
       <c r="N37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O37" t="b">
         <v>0</v>
@@ -2429,22 +2429,22 @@
         <v>113540</v>
       </c>
       <c r="I38" t="n">
-        <v>0.00102166637308438</v>
+        <v>0.0235355731401993</v>
       </c>
       <c r="J38" t="n">
-        <v>0.000844293898379367</v>
+        <v>0.0194421511101324</v>
       </c>
       <c r="K38" t="n">
-        <v>0.00122526665218281</v>
+        <v>0.0282389041012529</v>
       </c>
       <c r="L38" t="n">
-        <v>106</v>
+        <v>203</v>
       </c>
       <c r="M38" t="n">
-        <v>0.000933591685749516</v>
+        <v>0.178791615289766</v>
       </c>
       <c r="N38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O38" t="b">
         <v>0</v>
@@ -2476,19 +2476,19 @@
         <v>92874</v>
       </c>
       <c r="I39" t="n">
-        <v>0.00077524387880354</v>
+        <v>0.0197262489321322</v>
       </c>
       <c r="J39" t="n">
-        <v>0.000606628490147809</v>
+        <v>0.0154313568195835</v>
       </c>
       <c r="K39" t="n">
-        <v>0.000976193210741161</v>
+        <v>0.0248487354700057</v>
       </c>
       <c r="L39" t="n">
-        <v>92</v>
+        <v>172</v>
       </c>
       <c r="M39" t="n">
-        <v>0.000990589400693413</v>
+        <v>0.18519714882529</v>
       </c>
       <c r="N39" t="b">
         <v>0</v>
@@ -2523,19 +2523,19 @@
         <v>45157</v>
       </c>
       <c r="I40" t="n">
-        <v>0.000155014726399008</v>
+        <v>0.00384947926844576</v>
       </c>
       <c r="J40" t="n">
-        <v>0.0000623261582610724</v>
+        <v>0.00154755291274501</v>
       </c>
       <c r="K40" t="n">
-        <v>0.000319363332866307</v>
+        <v>0.00793330149319859</v>
       </c>
       <c r="L40" t="n">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="M40" t="n">
-        <v>0.000708638749252608</v>
+        <v>0.126226277210621</v>
       </c>
       <c r="N40" t="b">
         <v>0</v>
@@ -2570,19 +2570,19 @@
         <v>48845</v>
       </c>
       <c r="I41" t="n">
-        <v>0.000368512642030914</v>
+        <v>0.0103122249100067</v>
       </c>
       <c r="J41" t="n">
-        <v>0.000218418105234153</v>
+        <v>0.00611089685283511</v>
       </c>
       <c r="K41" t="n">
-        <v>0.000582346561326608</v>
+        <v>0.0163015182315711</v>
       </c>
       <c r="L41" t="n">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="M41" t="n">
-        <v>0.000716552359504555</v>
+        <v>0.139215886989456</v>
       </c>
       <c r="N41" t="b">
         <v>0</v>
@@ -2623,13 +2623,13 @@
         <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>0.000279400355503223</v>
+        <v>0.00812957105992258</v>
       </c>
       <c r="L42" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M42" t="n">
-        <v>0.000303007347928187</v>
+        <v>0.0530262858874328</v>
       </c>
       <c r="N42" t="b">
         <v>0</v>
@@ -2664,19 +2664,19 @@
         <v>85472</v>
       </c>
       <c r="I43" t="n">
-        <v>0.000386091351553725</v>
+        <v>0.0219381104885583</v>
       </c>
       <c r="J43" t="n">
-        <v>0.000265781957557443</v>
+        <v>0.0151009535149207</v>
       </c>
       <c r="K43" t="n">
-        <v>0.000542173476563157</v>
+        <v>0.0308102600306235</v>
       </c>
       <c r="L43" t="n">
-        <v>122</v>
+        <v>202</v>
       </c>
       <c r="M43" t="n">
-        <v>0.0014273680269562</v>
+        <v>0.236334706102583</v>
       </c>
       <c r="N43" t="b">
         <v>0</v>
@@ -2711,19 +2711,19 @@
         <v>74800</v>
       </c>
       <c r="I44" t="n">
-        <v>0.000481283422459893</v>
+        <v>0.0175611044917311</v>
       </c>
       <c r="J44" t="n">
-        <v>0.00033710704624923</v>
+        <v>0.0122986995679106</v>
       </c>
       <c r="K44" t="n">
-        <v>0.000666237483028853</v>
+        <v>0.0243146652263116</v>
       </c>
       <c r="L44" t="n">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="M44" t="n">
-        <v>0.000935828877005348</v>
+        <v>0.17379679144385</v>
       </c>
       <c r="N44" t="b">
         <v>0</v>
@@ -2758,19 +2758,19 @@
         <v>165442</v>
       </c>
       <c r="I45" t="n">
-        <v>0.000997328368854342</v>
+        <v>0.0385047191563009</v>
       </c>
       <c r="J45" t="n">
-        <v>0.000851016053538101</v>
+        <v>0.0328512508921773</v>
       </c>
       <c r="K45" t="n">
-        <v>0.00116155503104365</v>
+        <v>0.0448527589403779</v>
       </c>
       <c r="L45" t="n">
-        <v>296</v>
+        <v>594</v>
       </c>
       <c r="M45" t="n">
-        <v>0.00178914664958112</v>
+        <v>0.359038212787563</v>
       </c>
       <c r="N45" t="b">
         <v>0</v>
@@ -2805,19 +2805,19 @@
         <v>88735</v>
       </c>
       <c r="I46" t="n">
-        <v>0.000270468248154618</v>
+        <v>0.0113577853696363</v>
       </c>
       <c r="J46" t="n">
-        <v>0.000173301554163952</v>
+        <v>0.0072769108742162</v>
       </c>
       <c r="K46" t="n">
-        <v>0.000402408759438089</v>
+        <v>0.0169004776103161</v>
       </c>
       <c r="L46" t="n">
-        <v>53</v>
+        <v>102</v>
       </c>
       <c r="M46" t="n">
-        <v>0.000597284048008114</v>
+        <v>0.114949005465713</v>
       </c>
       <c r="N46" t="b">
         <v>0</v>
@@ -2852,19 +2852,19 @@
         <v>90416</v>
       </c>
       <c r="I47" t="n">
-        <v>0.000420279596531587</v>
+        <v>0.0169251270763115</v>
       </c>
       <c r="J47" t="n">
-        <v>0.000297431484907795</v>
+        <v>0.01197664306564</v>
       </c>
       <c r="K47" t="n">
-        <v>0.000576821415390172</v>
+        <v>0.0232328284613001</v>
       </c>
       <c r="L47" t="n">
-        <v>61</v>
+        <v>119</v>
       </c>
       <c r="M47" t="n">
-        <v>0.000674659352327022</v>
+        <v>0.131613873650681</v>
       </c>
       <c r="N47" t="b">
         <v>0</v>
@@ -2899,19 +2899,19 @@
         <v>86847</v>
       </c>
       <c r="I48" t="n">
-        <v>0.000598754130827778</v>
+        <v>0.0230052754712556</v>
       </c>
       <c r="J48" t="n">
-        <v>0.000447209546296734</v>
+        <v>0.0171802453100389</v>
       </c>
       <c r="K48" t="n">
-        <v>0.000785113184277431</v>
+        <v>0.0301713774509772</v>
       </c>
       <c r="L48" t="n">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="M48" t="n">
-        <v>0.000713899155986966</v>
+        <v>0.133568229184658</v>
       </c>
       <c r="N48" t="b">
         <v>0</v>
@@ -2946,19 +2946,19 @@
         <v>78865</v>
       </c>
       <c r="I49" t="n">
-        <v>0.000278957712546757</v>
+        <v>0.0147102222277732</v>
       </c>
       <c r="J49" t="n">
-        <v>0.000174829308383306</v>
+        <v>0.00921866570187686</v>
       </c>
       <c r="K49" t="n">
-        <v>0.000422315049111832</v>
+        <v>0.0222722808782927</v>
       </c>
       <c r="L49" t="n">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="M49" t="n">
-        <v>0.000646674697267482</v>
+        <v>0.106511126608762</v>
       </c>
       <c r="N49" t="b">
         <v>0</v>
@@ -2993,19 +2993,19 @@
         <v>83855</v>
       </c>
       <c r="I50" t="n">
-        <v>0.000727446186870193</v>
+        <v>0.0315981873500525</v>
       </c>
       <c r="J50" t="n">
-        <v>0.000556482962911442</v>
+        <v>0.0241686663711455</v>
       </c>
       <c r="K50" t="n">
-        <v>0.000934338340431995</v>
+        <v>0.0405926586045002</v>
       </c>
       <c r="L50" t="n">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="M50" t="n">
-        <v>0.00096595313338501</v>
+        <v>0.182457814083835</v>
       </c>
       <c r="N50" t="b">
         <v>0</v>
@@ -3040,19 +3040,19 @@
         <v>82752</v>
       </c>
       <c r="I51" t="n">
-        <v>0.000737142304717711</v>
+        <v>0.0272124650574152</v>
       </c>
       <c r="J51" t="n">
-        <v>0.000563900912946114</v>
+        <v>0.0208135404302072</v>
       </c>
       <c r="K51" t="n">
-        <v>0.000946790813783682</v>
+        <v>0.0349598305068229</v>
       </c>
       <c r="L51" t="n">
-        <v>82</v>
+        <v>154</v>
       </c>
       <c r="M51" t="n">
-        <v>0.000990912606341841</v>
+        <v>0.186098221191029</v>
       </c>
       <c r="N51" t="b">
         <v>0</v>
@@ -3087,19 +3087,19 @@
         <v>97236</v>
       </c>
       <c r="I52" t="n">
-        <v>0.000174832366613189</v>
+        <v>0.013909881093434</v>
       </c>
       <c r="J52" t="n">
-        <v>0.000101849489512751</v>
+        <v>0.00810308852559703</v>
       </c>
       <c r="K52" t="n">
-        <v>0.000279908846390176</v>
+        <v>0.0222710663883377</v>
       </c>
       <c r="L52" t="n">
-        <v>33</v>
+        <v>112</v>
       </c>
       <c r="M52" t="n">
-        <v>0.000339380476366778</v>
+        <v>0.115183676827512</v>
       </c>
       <c r="N52" t="b">
         <v>0</v>
@@ -3134,19 +3134,19 @@
         <v>94672</v>
       </c>
       <c r="I53" t="n">
-        <v>0.000359134696636809</v>
+        <v>0.0156865953710427</v>
       </c>
       <c r="J53" t="n">
-        <v>0.000248723637324422</v>
+        <v>0.0108630401817616</v>
       </c>
       <c r="K53" t="n">
-        <v>0.000501818927864606</v>
+        <v>0.0219217216842164</v>
       </c>
       <c r="L53" t="n">
-        <v>35</v>
+        <v>171</v>
       </c>
       <c r="M53" t="n">
-        <v>0.000369697481832009</v>
+        <v>0.180623626837925</v>
       </c>
       <c r="N53" t="b">
         <v>0</v>
@@ -3181,19 +3181,19 @@
         <v>130652</v>
       </c>
       <c r="I54" t="n">
-        <v>0.000742430272785721</v>
+        <v>0.0282064996113581</v>
       </c>
       <c r="J54" t="n">
-        <v>0.000602100898030478</v>
+        <v>0.0228719878845399</v>
       </c>
       <c r="K54" t="n">
-        <v>0.000905628024108873</v>
+        <v>0.0344126244765838</v>
       </c>
       <c r="L54" t="n">
-        <v>110</v>
+        <v>218</v>
       </c>
       <c r="M54" t="n">
-        <v>0.000841931237179683</v>
+        <v>0.166855463368337</v>
       </c>
       <c r="N54" t="b">
         <v>0</v>
@@ -3228,19 +3228,19 @@
         <v>107664</v>
       </c>
       <c r="I55" t="n">
-        <v>0.000900951107148165</v>
+        <v>0.0182796023551768</v>
       </c>
       <c r="J55" t="n">
-        <v>0.000730669505179971</v>
+        <v>0.014817334169937</v>
       </c>
       <c r="K55" t="n">
-        <v>0.00109897504683798</v>
+        <v>0.0223111345908309</v>
       </c>
       <c r="L55" t="n">
-        <v>102</v>
+        <v>162</v>
       </c>
       <c r="M55" t="n">
-        <v>0.000947391885867142</v>
+        <v>0.150468123049487</v>
       </c>
       <c r="N55" t="b">
         <v>0</v>
@@ -3275,19 +3275,19 @@
         <v>104891</v>
       </c>
       <c r="I56" t="n">
-        <v>0.000762696513523563</v>
+        <v>0.0244357388599961</v>
       </c>
       <c r="J56" t="n">
-        <v>0.000604815783723289</v>
+        <v>0.0193738404396642</v>
       </c>
       <c r="K56" t="n">
-        <v>0.000949153282571058</v>
+        <v>0.030416875346045</v>
       </c>
       <c r="L56" t="n">
-        <v>99</v>
+        <v>189</v>
       </c>
       <c r="M56" t="n">
-        <v>0.000943836935485409</v>
+        <v>0.180187051319942</v>
       </c>
       <c r="N56" t="b">
         <v>0</v>
@@ -3322,19 +3322,19 @@
         <v>89610</v>
       </c>
       <c r="I57" t="n">
-        <v>0.00088159803593349</v>
+        <v>0.0381540489179008</v>
       </c>
       <c r="J57" t="n">
-        <v>0.000698029673456002</v>
+        <v>0.0302049178138576</v>
       </c>
       <c r="K57" t="n">
-        <v>0.00109861489022478</v>
+        <v>0.0475556200361264</v>
       </c>
       <c r="L57" t="n">
-        <v>166</v>
+        <v>330</v>
       </c>
       <c r="M57" t="n">
-        <v>0.00185247182234126</v>
+        <v>0.368262470706394</v>
       </c>
       <c r="N57" t="b">
         <v>0</v>
@@ -3369,19 +3369,19 @@
         <v>93468</v>
       </c>
       <c r="I58" t="n">
-        <v>0.00057773783540891</v>
+        <v>0.0135905120390037</v>
       </c>
       <c r="J58" t="n">
-        <v>0.000434043316032029</v>
+        <v>0.010207408756539</v>
       </c>
       <c r="K58" t="n">
-        <v>0.000753756179486365</v>
+        <v>0.0177379079046336</v>
       </c>
       <c r="L58" t="n">
-        <v>60</v>
+        <v>111</v>
       </c>
       <c r="M58" t="n">
-        <v>0.000641930928232122</v>
+        <v>0.118757221722943</v>
       </c>
       <c r="N58" t="b">
         <v>0</v>
@@ -3416,19 +3416,19 @@
         <v>97469</v>
       </c>
       <c r="I59" t="n">
-        <v>0.000482204598385128</v>
+        <v>0.0120747618647055</v>
       </c>
       <c r="J59" t="n">
-        <v>0.000354326645038761</v>
+        <v>0.0088706635948277</v>
       </c>
       <c r="K59" t="n">
-        <v>0.000641178902906048</v>
+        <v>0.0160604936853504</v>
       </c>
       <c r="L59" t="n">
-        <v>74</v>
+        <v>135</v>
       </c>
       <c r="M59" t="n">
-        <v>0.000759215750648924</v>
+        <v>0.138505576131898</v>
       </c>
       <c r="N59" t="b">
         <v>0</v>
@@ -3463,19 +3463,19 @@
         <v>86839</v>
       </c>
       <c r="I60" t="n">
-        <v>0.000944276189269798</v>
+        <v>0.0249332915294612</v>
       </c>
       <c r="J60" t="n">
-        <v>0.000751079144831079</v>
+        <v>0.0198258421561042</v>
       </c>
       <c r="K60" t="n">
-        <v>0.00117196219696103</v>
+        <v>0.0309575154830267</v>
       </c>
       <c r="L60" t="n">
-        <v>86</v>
+        <v>162</v>
       </c>
       <c r="M60" t="n">
-        <v>0.00099033844240491</v>
+        <v>0.186552125197204</v>
       </c>
       <c r="N60" t="b">
         <v>0</v>
@@ -3510,19 +3510,19 @@
         <v>95425</v>
       </c>
       <c r="I61" t="n">
-        <v>0.00130992926381975</v>
+        <v>0.0258513739132753</v>
       </c>
       <c r="J61" t="n">
-        <v>0.00109048761395647</v>
+        <v>0.021505529559729</v>
       </c>
       <c r="K61" t="n">
-        <v>0.00156052582737021</v>
+        <v>0.0308229213473843</v>
       </c>
       <c r="L61" t="n">
-        <v>141</v>
+        <v>269</v>
       </c>
       <c r="M61" t="n">
-        <v>0.00147760020958868</v>
+        <v>0.281896777574011</v>
       </c>
       <c r="N61" t="b">
         <v>0</v>
@@ -3557,19 +3557,19 @@
         <v>92988</v>
       </c>
       <c r="I62" t="n">
-        <v>0.000871080139372822</v>
+        <v>0.0174286698746649</v>
       </c>
       <c r="J62" t="n">
-        <v>0.00069182168635884</v>
+        <v>0.0138345466175399</v>
       </c>
       <c r="K62" t="n">
-        <v>0.00108255851901629</v>
+        <v>0.0216748145327035</v>
       </c>
       <c r="L62" t="n">
-        <v>89</v>
+        <v>168</v>
       </c>
       <c r="M62" t="n">
-        <v>0.000957112745730632</v>
+        <v>0.1806684733514</v>
       </c>
       <c r="N62" t="b">
         <v>0</v>
@@ -3604,19 +3604,19 @@
         <v>119733</v>
       </c>
       <c r="I63" t="n">
-        <v>0.00101058187801191</v>
+        <v>0.0214234935681378</v>
       </c>
       <c r="J63" t="n">
-        <v>0.000838622692860169</v>
+        <v>0.0177700859491449</v>
       </c>
       <c r="K63" t="n">
-        <v>0.00120739746717335</v>
+        <v>0.0256098167985612</v>
       </c>
       <c r="L63" t="n">
-        <v>218</v>
+        <v>435</v>
       </c>
       <c r="M63" t="n">
-        <v>0.00182071776369088</v>
+        <v>0.363308361103455</v>
       </c>
       <c r="N63" t="b">
         <v>0</v>
@@ -3651,19 +3651,19 @@
         <v>78199</v>
       </c>
       <c r="I64" t="n">
-        <v>0.000601030703717439</v>
+        <v>0.0409873116805308</v>
       </c>
       <c r="J64" t="n">
-        <v>0.000441647137423673</v>
+        <v>0.030115808540355</v>
       </c>
       <c r="K64" t="n">
-        <v>0.000799164205526948</v>
+        <v>0.0545054177265182</v>
       </c>
       <c r="L64" t="n">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="M64" t="n">
-        <v>0.000652182252969987</v>
+        <v>0.106139464699037</v>
       </c>
       <c r="N64" t="b">
         <v>0</v>
@@ -3698,22 +3698,22 @@
         <v>76521</v>
       </c>
       <c r="I65" t="n">
-        <v>0.001163079416108</v>
+        <v>0.037473005012722</v>
       </c>
       <c r="J65" t="n">
-        <v>0.000934149173495769</v>
+        <v>0.030088999724761</v>
       </c>
       <c r="K65" t="n">
-        <v>0.00143107734093384</v>
+        <v>0.0461234073139839</v>
       </c>
       <c r="L65" t="n">
-        <v>71</v>
+        <v>133</v>
       </c>
       <c r="M65" t="n">
-        <v>0.000927849871277166</v>
+        <v>0.173808497013892</v>
       </c>
       <c r="N65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O65" t="b">
         <v>0</v>
@@ -3745,22 +3745,22 @@
         <v>144433</v>
       </c>
       <c r="I66" t="n">
-        <v>0.00101084932113852</v>
+        <v>0.0380563213307327</v>
       </c>
       <c r="J66" t="n">
-        <v>0.000853598799265054</v>
+        <v>0.0321311532690353</v>
       </c>
       <c r="K66" t="n">
-        <v>0.00118865182653127</v>
+        <v>0.0447586467653664</v>
       </c>
       <c r="L66" t="n">
-        <v>138</v>
+        <v>261</v>
       </c>
       <c r="M66" t="n">
-        <v>0.00095546031724052</v>
+        <v>0.180706625217229</v>
       </c>
       <c r="N66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O66" t="b">
         <v>0</v>
@@ -3792,19 +3792,19 @@
         <v>69495</v>
       </c>
       <c r="I67" t="n">
-        <v>0.000402906683934096</v>
+        <v>0.0241326633153669</v>
       </c>
       <c r="J67" t="n">
-        <v>0.000267744737073916</v>
+        <v>0.016035790198901</v>
       </c>
       <c r="K67" t="n">
-        <v>0.000582260101280929</v>
+        <v>0.0348794982986761</v>
       </c>
       <c r="L67" t="n">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="M67" t="n">
-        <v>0.000532412403770055</v>
+        <v>0.102165623426146</v>
       </c>
       <c r="N67" t="b">
         <v>0</v>
@@ -3839,19 +3839,19 @@
         <v>70360</v>
       </c>
       <c r="I68" t="n">
-        <v>0.00027003979533826</v>
+        <v>0.0160899658692616</v>
       </c>
       <c r="J68" t="n">
-        <v>0.000162589177769346</v>
+        <v>0.00968713617273247</v>
       </c>
       <c r="K68" t="n">
-        <v>0.000421668612710202</v>
+        <v>0.0251271488599988</v>
       </c>
       <c r="L68" t="n">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="M68" t="n">
-        <v>0.000483229107447413</v>
+        <v>0.0938032973280273</v>
       </c>
       <c r="N68" t="b">
         <v>0</v>
@@ -3886,19 +3886,19 @@
         <v>86993</v>
       </c>
       <c r="I69" t="n">
-        <v>0.000827652799650547</v>
+        <v>0.0345282648333177</v>
       </c>
       <c r="J69" t="n">
-        <v>0.00064764193925293</v>
+        <v>0.0270143394306296</v>
       </c>
       <c r="K69" t="n">
-        <v>0.00104217985262489</v>
+        <v>0.0434868372970648</v>
       </c>
       <c r="L69" t="n">
-        <v>76</v>
+        <v>149</v>
       </c>
       <c r="M69" t="n">
-        <v>0.000873633510742244</v>
+        <v>0.171278148816571</v>
       </c>
       <c r="N69" t="b">
         <v>0</v>
@@ -3933,19 +3933,19 @@
         <v>75605</v>
       </c>
       <c r="I70" t="n">
-        <v>0.000343892599695787</v>
+        <v>0.0192080693716811</v>
       </c>
       <c r="J70" t="n">
-        <v>0.000224653973762923</v>
+        <v>0.0125471559679172</v>
       </c>
       <c r="K70" t="n">
-        <v>0.000503842027797408</v>
+        <v>0.0281452580095622</v>
       </c>
       <c r="L70" t="n">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="M70" t="n">
-        <v>0.000529065537993519</v>
+        <v>0.100522452218769</v>
       </c>
       <c r="N70" t="b">
         <v>0</v>
@@ -3980,19 +3980,19 @@
         <v>75439</v>
       </c>
       <c r="I71" t="n">
-        <v>0.000450695263723008</v>
+        <v>0.022446981263569</v>
       </c>
       <c r="J71" t="n">
-        <v>0.000312139132411793</v>
+        <v>0.0155447145929661</v>
       </c>
       <c r="K71" t="n">
-        <v>0.000629745053397079</v>
+        <v>0.0313690927627339</v>
       </c>
       <c r="L71" t="n">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="M71" t="n">
-        <v>0.000477206749824361</v>
+        <v>0.0927902013547369</v>
       </c>
       <c r="N71" t="b">
         <v>0</v>
@@ -4027,22 +4027,22 @@
         <v>85442</v>
       </c>
       <c r="I72" t="n">
-        <v>0.000912899978933077</v>
+        <v>0.0325007299458898</v>
       </c>
       <c r="J72" t="n">
-        <v>0.000721674365213976</v>
+        <v>0.0256877097070365</v>
       </c>
       <c r="K72" t="n">
-        <v>0.00113921147376073</v>
+        <v>0.0405681693165143</v>
       </c>
       <c r="L72" t="n">
-        <v>75</v>
+        <v>147</v>
       </c>
       <c r="M72" t="n">
-        <v>0.000877788441281805</v>
+        <v>0.172046534491234</v>
       </c>
       <c r="N72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O72" t="b">
         <v>0</v>
@@ -4074,19 +4074,19 @@
         <v>72471</v>
       </c>
       <c r="I73" t="n">
-        <v>0.000289771080846132</v>
+        <v>0.0202397123901458</v>
       </c>
       <c r="J73" t="n">
-        <v>0.000179381530774791</v>
+        <v>0.0125287333113717</v>
       </c>
       <c r="K73" t="n">
-        <v>0.000442911953492997</v>
+        <v>0.0309389179276725</v>
       </c>
       <c r="L73" t="n">
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="M73" t="n">
-        <v>0.000772722882256351</v>
+        <v>0.15040498958204</v>
       </c>
       <c r="N73" t="b">
         <v>0</v>
@@ -4121,19 +4121,19 @@
         <v>77697</v>
       </c>
       <c r="I74" t="n">
-        <v>0.000373244784225903</v>
+        <v>0.0233743473385365</v>
       </c>
       <c r="J74" t="n">
-        <v>0.000249981690721879</v>
+        <v>0.0156540508534198</v>
       </c>
       <c r="K74" t="n">
-        <v>0.000535998135967275</v>
+        <v>0.0335702507749955</v>
       </c>
       <c r="L74" t="n">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="M74" t="n">
-        <v>0.000476208862633049</v>
+        <v>0.0926676705664311</v>
       </c>
       <c r="N74" t="b">
         <v>0</v>
@@ -4168,19 +4168,19 @@
         <v>120845</v>
       </c>
       <c r="I75" t="n">
-        <v>0.000645454921593777</v>
+        <v>0.0226971955687063</v>
       </c>
       <c r="J75" t="n">
-        <v>0.000510237729134833</v>
+        <v>0.0179397910617122</v>
       </c>
       <c r="K75" t="n">
-        <v>0.000805492461282142</v>
+        <v>0.0283300616822594</v>
       </c>
       <c r="L75" t="n">
-        <v>103</v>
+        <v>203</v>
       </c>
       <c r="M75" t="n">
-        <v>0.00085233149902768</v>
+        <v>0.167983780876329</v>
       </c>
       <c r="N75" t="b">
         <v>0</v>
@@ -4215,19 +4215,19 @@
         <v>85789</v>
       </c>
       <c r="I76" t="n">
-        <v>0.00022147361549849</v>
+        <v>0.0108417693097412</v>
       </c>
       <c r="J76" t="n">
-        <v>0.000133346683278579</v>
+        <v>0.00652733726747841</v>
       </c>
       <c r="K76" t="n">
-        <v>0.000345836975016334</v>
+        <v>0.0169314281341736</v>
       </c>
       <c r="L76" t="n">
-        <v>41</v>
+        <v>99</v>
       </c>
       <c r="M76" t="n">
-        <v>0.000477916749233585</v>
+        <v>0.115399410180792</v>
       </c>
       <c r="N76" t="b">
         <v>0</v>
@@ -4256,25 +4256,25 @@
         <v>21</v>
       </c>
       <c r="G77" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="H77" t="n">
         <v>85848</v>
       </c>
       <c r="I77" t="n">
-        <v>0.000477588295592209</v>
+        <v>0.0167428746951768</v>
       </c>
       <c r="J77" t="n">
-        <v>0.000342746724331433</v>
+        <v>0.0122566137427708</v>
       </c>
       <c r="K77" t="n">
-        <v>0.000647847273809177</v>
+        <v>0.0223359862769231</v>
       </c>
       <c r="L77" t="n">
-        <v>82</v>
+        <v>160</v>
       </c>
       <c r="M77" t="n">
-        <v>0.000955176591184419</v>
+        <v>0.186375920231106</v>
       </c>
       <c r="N77" t="b">
         <v>0</v>
@@ -4309,22 +4309,22 @@
         <v>188739</v>
       </c>
       <c r="I78" t="n">
-        <v>0.000524533880120166</v>
+        <v>0.0193175064415262</v>
       </c>
       <c r="J78" t="n">
-        <v>0.000426335064640626</v>
+        <v>0.0156995026381077</v>
       </c>
       <c r="K78" t="n">
-        <v>0.000638564753098869</v>
+        <v>0.0235199454658413</v>
       </c>
       <c r="L78" t="n">
-        <v>30</v>
+        <v>310</v>
       </c>
       <c r="M78" t="n">
-        <v>0.000158949660642475</v>
+        <v>0.16424798266389</v>
       </c>
       <c r="N78" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O78" t="b">
         <v>0</v>
@@ -4356,19 +4356,19 @@
         <v>73903</v>
       </c>
       <c r="I79" t="n">
-        <v>0.000405937512685547</v>
+        <v>0.0239060554744223</v>
       </c>
       <c r="J79" t="n">
-        <v>0.000273900568166008</v>
+        <v>0.0161291000177226</v>
       </c>
       <c r="K79" t="n">
-        <v>0.000579450748431021</v>
+        <v>0.03412846818393</v>
       </c>
       <c r="L79" t="n">
-        <v>39</v>
+        <v>75</v>
       </c>
       <c r="M79" t="n">
-        <v>0.000527718766491211</v>
+        <v>0.101484378171387</v>
       </c>
       <c r="N79" t="b">
         <v>0</v>
@@ -4403,19 +4403,19 @@
         <v>68924</v>
       </c>
       <c r="I80" t="n">
-        <v>0.000290174685160467</v>
+        <v>0.0148160469152229</v>
       </c>
       <c r="J80" t="n">
-        <v>0.000177254959430995</v>
+        <v>0.00904984651451865</v>
       </c>
       <c r="K80" t="n">
-        <v>0.000448115867401899</v>
+        <v>0.022883204343539</v>
       </c>
       <c r="L80" t="n">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="M80" t="n">
-        <v>0.00047878823051477</v>
+        <v>0.0943067726771517</v>
       </c>
       <c r="N80" t="b">
         <v>0</v>
@@ -4450,19 +4450,19 @@
         <v>88476</v>
       </c>
       <c r="I81" t="n">
-        <v>0.0007685700076857</v>
+        <v>0.0421088154853624</v>
       </c>
       <c r="J81" t="n">
-        <v>0.000596872574298635</v>
+        <v>0.0326981434050756</v>
       </c>
       <c r="K81" t="n">
-        <v>0.000974245360945258</v>
+        <v>0.0533854950789827</v>
       </c>
       <c r="L81" t="n">
-        <v>164</v>
+        <v>326</v>
       </c>
       <c r="M81" t="n">
-        <v>0.0018536100185361</v>
+        <v>0.368461503684615</v>
       </c>
       <c r="N81" t="b">
         <v>0</v>
@@ -4497,22 +4497,22 @@
         <v>94639</v>
       </c>
       <c r="I82" t="n">
-        <v>0.00161666966049937</v>
+        <v>0.042256088685131</v>
       </c>
       <c r="J82" t="n">
-        <v>0.0013708138692875</v>
+        <v>0.0358151806679679</v>
       </c>
       <c r="K82" t="n">
-        <v>0.00189383353045214</v>
+        <v>0.0495248246194218</v>
       </c>
       <c r="L82" t="n">
-        <v>140</v>
+        <v>267</v>
       </c>
       <c r="M82" t="n">
-        <v>0.00147930557169877</v>
+        <v>0.282124705459694</v>
       </c>
       <c r="N82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O82" t="b">
         <v>0</v>
@@ -4544,22 +4544,22 @@
         <v>95271</v>
       </c>
       <c r="I83" t="n">
-        <v>0.00107063009730138</v>
+        <v>0.0274684595600509</v>
       </c>
       <c r="J83" t="n">
-        <v>0.000873052617013981</v>
+        <v>0.0223917809917299</v>
       </c>
       <c r="K83" t="n">
-        <v>0.0012995230228996</v>
+        <v>0.0333549981274794</v>
       </c>
       <c r="L83" t="n">
-        <v>91</v>
+        <v>172</v>
       </c>
       <c r="M83" t="n">
-        <v>0.00095516998876888</v>
+        <v>0.180537624250821</v>
       </c>
       <c r="N83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O83" t="b">
         <v>0</v>
@@ -4591,22 +4591,22 @@
         <v>93457</v>
       </c>
       <c r="I84" t="n">
-        <v>0.00102721037482479</v>
+        <v>0.0295646949267645</v>
       </c>
       <c r="J84" t="n">
-        <v>0.000832120468651998</v>
+        <v>0.023943175743506</v>
       </c>
       <c r="K84" t="n">
-        <v>0.00125425716336669</v>
+        <v>0.0361118022338689</v>
       </c>
       <c r="L84" t="n">
-        <v>68</v>
+        <v>138</v>
       </c>
       <c r="M84" t="n">
-        <v>0.000727607348834223</v>
+        <v>0.147661491381063</v>
       </c>
       <c r="N84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O84" t="b">
         <v>0</v>
@@ -4638,19 +4638,19 @@
         <v>14236</v>
       </c>
       <c r="I85" t="n">
-        <v>0.000491711154818769</v>
+        <v>0.053602431322814</v>
       </c>
       <c r="J85" t="n">
-        <v>0.000197715510313667</v>
+        <v>0.0215535354960599</v>
       </c>
       <c r="K85" t="n">
-        <v>0.0010128488051655</v>
+        <v>0.110430069440483</v>
       </c>
       <c r="L85" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="M85" t="n">
-        <v>0.000491711154818769</v>
+        <v>0.126440011239112</v>
       </c>
       <c r="N85" t="b">
         <v>0</v>
@@ -4685,19 +4685,19 @@
         <v>15246</v>
       </c>
       <c r="I86" t="n">
-        <v>0.000262363898727535</v>
+        <v>0.0254830325871382</v>
       </c>
       <c r="J86" t="n">
-        <v>0.0000714898107250228</v>
+        <v>0.00694375942169774</v>
       </c>
       <c r="K86" t="n">
-        <v>0.000671618288535347</v>
+        <v>0.0652435090942769</v>
       </c>
       <c r="L86" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="M86" t="n">
-        <v>0.000852682670864489</v>
+        <v>0.157418339236521</v>
       </c>
       <c r="N86" t="b">
         <v>0</v>
@@ -4732,19 +4732,19 @@
         <v>14766</v>
       </c>
       <c r="I87" t="n">
-        <v>0.00128673980766626</v>
+        <v>0.172367405668943</v>
       </c>
       <c r="J87" t="n">
-        <v>0.000774873608921922</v>
+        <v>0.103802529429356</v>
       </c>
       <c r="K87" t="n">
-        <v>0.00200867749519074</v>
+        <v>0.269104656469841</v>
       </c>
       <c r="L87" t="n">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="M87" t="n">
-        <v>0.00203169443315725</v>
+        <v>0.386021942299878</v>
       </c>
       <c r="N87" t="b">
         <v>0</v>
@@ -4779,19 +4779,19 @@
         <v>90342</v>
       </c>
       <c r="I88" t="n">
-        <v>0.000719488167186912</v>
+        <v>0.0445094347884203</v>
       </c>
       <c r="J88" t="n">
-        <v>0.000555328304152614</v>
+        <v>0.0343508919468904</v>
       </c>
       <c r="K88" t="n">
-        <v>0.000916956136543967</v>
+        <v>0.0567326235826088</v>
       </c>
       <c r="L88" t="n">
-        <v>129</v>
+        <v>213</v>
       </c>
       <c r="M88" t="n">
-        <v>0.00142790728564787</v>
+        <v>0.235770737862788</v>
       </c>
       <c r="N88" t="b">
         <v>0</v>
@@ -4826,19 +4826,19 @@
         <v>92756</v>
       </c>
       <c r="I89" t="n">
-        <v>0.000582172581827591</v>
+        <v>0.0388844257519165</v>
       </c>
       <c r="J89" t="n">
-        <v>0.000437375279035535</v>
+        <v>0.0292109931786612</v>
       </c>
       <c r="K89" t="n">
-        <v>0.000759541538656539</v>
+        <v>0.0507366742463916</v>
       </c>
       <c r="L89" t="n">
-        <v>85</v>
+        <v>159</v>
       </c>
       <c r="M89" t="n">
-        <v>0.000916382767691578</v>
+        <v>0.171417482427013</v>
       </c>
       <c r="N89" t="b">
         <v>0</v>
@@ -4873,19 +4873,19 @@
         <v>82013</v>
       </c>
       <c r="I90" t="n">
-        <v>0.00119493251069952</v>
+        <v>0.0579404547564839</v>
       </c>
       <c r="J90" t="n">
-        <v>0.000970207150423397</v>
+        <v>0.0470359490640442</v>
       </c>
       <c r="K90" t="n">
-        <v>0.00145604968819546</v>
+        <v>0.0706167538148781</v>
       </c>
       <c r="L90" t="n">
-        <v>153</v>
+        <v>303</v>
       </c>
       <c r="M90" t="n">
-        <v>0.00186555789935742</v>
+        <v>0.369453623206077</v>
       </c>
       <c r="N90" t="b">
         <v>0</v>
@@ -4920,19 +4920,19 @@
         <v>86209</v>
       </c>
       <c r="I91" t="n">
-        <v>0.00121797028152513</v>
+        <v>0.0314533998424005</v>
       </c>
       <c r="J91" t="n">
-        <v>0.000996283756446448</v>
+        <v>0.0257188199710026</v>
       </c>
       <c r="K91" t="n">
-        <v>0.00147423818235448</v>
+        <v>0.0380890363700119</v>
       </c>
       <c r="L91" t="n">
-        <v>129</v>
+        <v>244</v>
       </c>
       <c r="M91" t="n">
-        <v>0.00149636348873087</v>
+        <v>0.283033093992507</v>
       </c>
       <c r="N91" t="b">
         <v>0</v>
@@ -4967,22 +4967,22 @@
         <v>80253</v>
       </c>
       <c r="I92" t="n">
-        <v>0.00120867755722528</v>
+        <v>0.0314569164166978</v>
       </c>
       <c r="J92" t="n">
-        <v>0.000980262003317467</v>
+        <v>0.0255025084728647</v>
       </c>
       <c r="K92" t="n">
-        <v>0.00147428811432859</v>
+        <v>0.0383878584223302</v>
       </c>
       <c r="L92" t="n">
-        <v>77</v>
+        <v>147</v>
       </c>
       <c r="M92" t="n">
-        <v>0.000959465689756146</v>
+        <v>0.18317072258981</v>
       </c>
       <c r="N92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O92" t="b">
         <v>0</v>
@@ -5014,22 +5014,22 @@
         <v>88225</v>
       </c>
       <c r="I93" t="n">
-        <v>0.00116746953811278</v>
+        <v>0.0315529668580529</v>
       </c>
       <c r="J93" t="n">
-        <v>0.000953023332936787</v>
+        <v>0.0257485711585276</v>
       </c>
       <c r="K93" t="n">
-        <v>0.00141572044110438</v>
+        <v>0.0382782560806413</v>
       </c>
       <c r="L93" t="n">
-        <v>65</v>
+        <v>131</v>
       </c>
       <c r="M93" t="n">
-        <v>0.000736752621139133</v>
+        <v>0.14848398979881</v>
       </c>
       <c r="N93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O93" t="b">
         <v>0</v>
@@ -5061,19 +5061,19 @@
         <v>95751</v>
       </c>
       <c r="I94" t="n">
-        <v>0.00134724441520193</v>
+        <v>0.043105871029757</v>
       </c>
       <c r="J94" t="n">
-        <v>0.00112492036362377</v>
+        <v>0.0359827787315746</v>
       </c>
       <c r="K94" t="n">
-        <v>0.00160060113462446</v>
+        <v>0.0512289493378014</v>
       </c>
       <c r="L94" t="n">
-        <v>142</v>
+        <v>270</v>
       </c>
       <c r="M94" t="n">
-        <v>0.00148301323223778</v>
+        <v>0.281981389228311</v>
       </c>
       <c r="N94" t="b">
         <v>0</v>
@@ -5108,22 +5108,22 @@
         <v>103296</v>
       </c>
       <c r="I95" t="n">
-        <v>0.000997134448574969</v>
+        <v>0.0318701130104025</v>
       </c>
       <c r="J95" t="n">
-        <v>0.0008139641070527</v>
+        <v>0.0260099495408038</v>
       </c>
       <c r="K95" t="n">
-        <v>0.00120918719621788</v>
+        <v>0.0386582940297078</v>
       </c>
       <c r="L95" t="n">
-        <v>98</v>
+        <v>186</v>
       </c>
       <c r="M95" t="n">
-        <v>0.000948729863692689</v>
+        <v>0.180065055762082</v>
       </c>
       <c r="N95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O95" t="b">
         <v>0</v>
@@ -5155,22 +5155,22 @@
         <v>95599</v>
       </c>
       <c r="I96" t="n">
-        <v>0.00085774955804977</v>
+        <v>0.0274096881064484</v>
       </c>
       <c r="J96" t="n">
-        <v>0.000682250007566387</v>
+        <v>0.021796987727406</v>
       </c>
       <c r="K96" t="n">
-        <v>0.00106458318533131</v>
+        <v>0.0340282451051463</v>
       </c>
       <c r="L96" t="n">
-        <v>69</v>
+        <v>141</v>
       </c>
       <c r="M96" t="n">
-        <v>0.00072176487201749</v>
+        <v>0.147491082542704</v>
       </c>
       <c r="N96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O96" t="b">
         <v>0</v>
@@ -5202,19 +5202,19 @@
         <v>85043</v>
       </c>
       <c r="I97" t="n">
-        <v>0.000670249168067919</v>
+        <v>0.0262701954085194</v>
       </c>
       <c r="J97" t="n">
-        <v>0.000507678471913464</v>
+        <v>0.0198953584175922</v>
       </c>
       <c r="K97" t="n">
-        <v>0.000868299501569192</v>
+        <v>0.034039555616521</v>
       </c>
       <c r="L97" t="n">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="M97" t="n">
-        <v>0.000964218101431041</v>
+        <v>0.152863845348824</v>
       </c>
       <c r="N97" t="b">
         <v>0</v>
@@ -5249,19 +5249,19 @@
         <v>89376</v>
       </c>
       <c r="I98" t="n">
-        <v>0.000615377730039384</v>
+        <v>0.0331551300758133</v>
       </c>
       <c r="J98" t="n">
-        <v>0.000463619320583697</v>
+        <v>0.0249762895101708</v>
       </c>
       <c r="K98" t="n">
-        <v>0.000800924354384835</v>
+        <v>0.0431579042145547</v>
       </c>
       <c r="L98" t="n">
-        <v>77</v>
+        <v>141</v>
       </c>
       <c r="M98" t="n">
-        <v>0.000861528822055138</v>
+        <v>0.157760472610097</v>
       </c>
       <c r="N98" t="b">
         <v>0</v>
@@ -5296,19 +5296,19 @@
         <v>88207</v>
       </c>
       <c r="I99" t="n">
-        <v>0.000362782999081706</v>
+        <v>0.0144135057618551</v>
       </c>
       <c r="J99" t="n">
-        <v>0.000248156121403831</v>
+        <v>0.00985837396906454</v>
       </c>
       <c r="K99" t="n">
-        <v>0.000512103102543127</v>
+        <v>0.0203490914297583</v>
       </c>
       <c r="L99" t="n">
-        <v>65</v>
+        <v>131</v>
       </c>
       <c r="M99" t="n">
-        <v>0.000736902966884714</v>
+        <v>0.148514290249073</v>
       </c>
       <c r="N99" t="b">
         <v>0</v>
@@ -5343,19 +5343,19 @@
         <v>78573</v>
       </c>
       <c r="I100" t="n">
-        <v>0.000458172654728724</v>
+        <v>0.0188765540075931</v>
       </c>
       <c r="J100" t="n">
-        <v>0.000320918481316657</v>
+        <v>0.0132202279677168</v>
       </c>
       <c r="K100" t="n">
-        <v>0.00063424821689273</v>
+        <v>0.0261352396850686</v>
       </c>
       <c r="L100" t="n">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="M100" t="n">
-        <v>0.000483626691102542</v>
+        <v>0.0954526364018174</v>
       </c>
       <c r="N100" t="b">
         <v>0</v>
@@ -5384,25 +5384,25 @@
         <v>21</v>
       </c>
       <c r="G101" t="n">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="H101" t="n">
         <v>72663</v>
       </c>
       <c r="I101" t="n">
-        <v>0.000550486492437692</v>
+        <v>0.038720926552352</v>
       </c>
       <c r="J101" t="n">
-        <v>0.000393303833721936</v>
+        <v>0.0306035114703714</v>
       </c>
       <c r="K101" t="n">
-        <v>0.000749531724770325</v>
+        <v>0.0483333530718642</v>
       </c>
       <c r="L101" t="n">
-        <v>70</v>
+        <v>137</v>
       </c>
       <c r="M101" t="n">
-        <v>0.000963351361765961</v>
+        <v>0.188541623659909</v>
       </c>
       <c r="N101" t="b">
         <v>0</v>
@@ -5437,19 +5437,19 @@
         <v>85830</v>
       </c>
       <c r="I102" t="n">
-        <v>0.000431084702318537</v>
+        <v>0.0173366531430819</v>
       </c>
       <c r="J102" t="n">
-        <v>0.00030354100674268</v>
+        <v>0.0122059852803971</v>
       </c>
       <c r="K102" t="n">
-        <v>0.000594145015703651</v>
+        <v>0.0238981938617693</v>
       </c>
       <c r="L102" t="n">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="M102" t="n">
-        <v>0.000512641267622044</v>
+        <v>0.0932075032040079</v>
       </c>
       <c r="N102" t="b">
         <v>0</v>
@@ -5484,19 +5484,19 @@
         <v>91644</v>
       </c>
       <c r="I103" t="n">
-        <v>0.000763825236785823</v>
+        <v>0.0240268801302244</v>
       </c>
       <c r="J103" t="n">
-        <v>0.000595486139194468</v>
+        <v>0.0187278064169064</v>
       </c>
       <c r="K103" t="n">
-        <v>0.000964950129572761</v>
+        <v>0.0303615433460644</v>
       </c>
       <c r="L103" t="n">
-        <v>136</v>
+        <v>259</v>
       </c>
       <c r="M103" t="n">
-        <v>0.00148400331718389</v>
+        <v>0.282615337610755</v>
       </c>
       <c r="N103" t="b">
         <v>0</v>
@@ -5525,25 +5525,25 @@
         <v>21</v>
       </c>
       <c r="G104" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="H104" t="n">
         <v>90133</v>
       </c>
       <c r="I104" t="n">
-        <v>0.000809914237848513</v>
+        <v>0.0285339416540302</v>
       </c>
       <c r="J104" t="n">
-        <v>0.000634895538168534</v>
+        <v>0.0226907198958314</v>
       </c>
       <c r="K104" t="n">
-        <v>0.00101823941712875</v>
+        <v>0.0354245816921393</v>
       </c>
       <c r="L104" t="n">
-        <v>86</v>
+        <v>167</v>
       </c>
       <c r="M104" t="n">
-        <v>0.00095414554047907</v>
+        <v>0.185281750302331</v>
       </c>
       <c r="N104" t="b">
         <v>0</v>
@@ -5578,19 +5578,19 @@
         <v>84982</v>
       </c>
       <c r="I105" t="n">
-        <v>0.000941375820762044</v>
+        <v>0.0271066256008985</v>
       </c>
       <c r="J105" t="n">
-        <v>0.000746520858671884</v>
+        <v>0.0214900358201436</v>
       </c>
       <c r="K105" t="n">
-        <v>0.00117148879414575</v>
+        <v>0.0337443469466338</v>
       </c>
       <c r="L105" t="n">
-        <v>158</v>
+        <v>313</v>
       </c>
       <c r="M105" t="n">
-        <v>0.00185921724600504</v>
+        <v>0.36831328987315</v>
       </c>
       <c r="N105" t="b">
         <v>0</v>
@@ -5625,19 +5625,19 @@
         <v>81327</v>
       </c>
       <c r="I106" t="n">
-        <v>0.000516433656719171</v>
+        <v>0.0176235365496633</v>
       </c>
       <c r="J106" t="n">
-        <v>0.000372224512867891</v>
+        <v>0.0127004176581919</v>
       </c>
       <c r="K106" t="n">
-        <v>0.000698004876521496</v>
+        <v>0.0238248876870244</v>
       </c>
       <c r="L106" t="n">
-        <v>117</v>
+        <v>193</v>
       </c>
       <c r="M106" t="n">
-        <v>0.00143863661514626</v>
+        <v>0.237313561301905</v>
       </c>
       <c r="N106" t="b">
         <v>0</v>
@@ -5672,19 +5672,19 @@
         <v>90230</v>
       </c>
       <c r="I107" t="n">
-        <v>0.000144076249584395</v>
+        <v>0.00530164679248969</v>
       </c>
       <c r="J107" t="n">
-        <v>0.0000767166938048236</v>
+        <v>0.00282282503900076</v>
       </c>
       <c r="K107" t="n">
-        <v>0.000246362172787062</v>
+        <v>0.00906652577954669</v>
       </c>
       <c r="L107" t="n">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="M107" t="n">
-        <v>0.000919871439654217</v>
+        <v>0.171783220658318</v>
       </c>
       <c r="N107" t="b">
         <v>0</v>
@@ -5719,19 +5719,19 @@
         <v>86777</v>
       </c>
       <c r="I108" t="n">
-        <v>0.000276570980789841</v>
+        <v>0.0104511839541715</v>
       </c>
       <c r="J108" t="n">
-        <v>0.000177212029854878</v>
+        <v>0.00669598219328942</v>
       </c>
       <c r="K108" t="n">
-        <v>0.000411487929987575</v>
+        <v>0.0155517026168617</v>
       </c>
       <c r="L108" t="n">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="M108" t="n">
-        <v>0.000610760915910898</v>
+        <v>0.124456941355428</v>
       </c>
       <c r="N108" t="b">
         <v>0</v>
@@ -5766,19 +5766,19 @@
         <v>81324</v>
       </c>
       <c r="I109" t="n">
-        <v>0.000454970242486843</v>
+        <v>0.0179551264344913</v>
       </c>
       <c r="J109" t="n">
-        <v>0.000320360635118755</v>
+        <v>0.0126413585751413</v>
       </c>
       <c r="K109" t="n">
-        <v>0.000627062567257197</v>
+        <v>0.0247509395655489</v>
       </c>
       <c r="L109" t="n">
-        <v>79</v>
+        <v>125</v>
       </c>
       <c r="M109" t="n">
-        <v>0.00097142295017461</v>
+        <v>0.153706163002312</v>
       </c>
       <c r="N109" t="b">
         <v>0</v>
@@ -5813,22 +5813,22 @@
         <v>175608</v>
       </c>
       <c r="I110" t="n">
-        <v>0.00104778825566033</v>
+        <v>0.0488230042682513</v>
       </c>
       <c r="J110" t="n">
-        <v>0.000901919667053552</v>
+        <v>0.0420211737294389</v>
       </c>
       <c r="K110" t="n">
-        <v>0.00121050998021754</v>
+        <v>0.0564130506850896</v>
       </c>
       <c r="L110" t="n">
-        <v>153</v>
+        <v>291</v>
       </c>
       <c r="M110" t="n">
-        <v>0.000871258712587126</v>
+        <v>0.165709990433238</v>
       </c>
       <c r="N110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O110" t="b">
         <v>0</v>
@@ -5860,19 +5860,19 @@
         <v>85449</v>
       </c>
       <c r="I111" t="n">
-        <v>0.000304275064658451</v>
+        <v>0.011919418482271</v>
       </c>
       <c r="J111" t="n">
-        <v>0.000198771898298977</v>
+        <v>0.0077858288836382</v>
       </c>
       <c r="K111" t="n">
-        <v>0.000445801912372867</v>
+        <v>0.017465986293656</v>
       </c>
       <c r="L111" t="n">
-        <v>53</v>
+        <v>107</v>
       </c>
       <c r="M111" t="n">
-        <v>0.000620253016419151</v>
+        <v>0.125220891994055</v>
       </c>
       <c r="N111" t="b">
         <v>0</v>
@@ -5907,19 +5907,19 @@
         <v>76031</v>
       </c>
       <c r="I112" t="n">
-        <v>0.000223593008115111</v>
+        <v>0.00769671616699978</v>
       </c>
       <c r="J112" t="n">
-        <v>0.000130256389707428</v>
+        <v>0.00448340660637157</v>
       </c>
       <c r="K112" t="n">
-        <v>0.000357970008217912</v>
+        <v>0.0123243135824689</v>
       </c>
       <c r="L112" t="n">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="M112" t="n">
-        <v>0.000486643605897594</v>
+        <v>0.0960134681906065</v>
       </c>
       <c r="N112" t="b">
         <v>0</v>
@@ -5948,25 +5948,25 @@
         <v>21</v>
       </c>
       <c r="G113" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="H113" t="n">
         <v>83186</v>
       </c>
       <c r="I113" t="n">
-        <v>0.000432765128747626</v>
+        <v>0.024343356125354</v>
       </c>
       <c r="J113" t="n">
-        <v>0.000303121207095192</v>
+        <v>0.0182860407527915</v>
       </c>
       <c r="K113" t="n">
-        <v>0.000599079515354983</v>
+        <v>0.0317663496039385</v>
       </c>
       <c r="L113" t="n">
-        <v>79</v>
+        <v>155</v>
       </c>
       <c r="M113" t="n">
-        <v>0.000949679032529512</v>
+        <v>0.186329430433006</v>
       </c>
       <c r="N113" t="b">
         <v>0</v>
@@ -6001,19 +6001,19 @@
         <v>85416</v>
       </c>
       <c r="I114" t="n">
-        <v>0.000421466704130374</v>
+        <v>0.0156243963734717</v>
       </c>
       <c r="J114" t="n">
-        <v>0.000295207010419518</v>
+        <v>0.0109424734349879</v>
       </c>
       <c r="K114" t="n">
-        <v>0.000583440301689997</v>
+        <v>0.0216327809733265</v>
       </c>
       <c r="L114" t="n">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="M114" t="n">
-        <v>0.000515125971714901</v>
+        <v>0.0924885267397209</v>
       </c>
       <c r="N114" t="b">
         <v>0</v>
@@ -6048,19 +6048,19 @@
         <v>92821</v>
       </c>
       <c r="I115" t="n">
-        <v>0.000215468482347745</v>
+        <v>0.00702945867265465</v>
       </c>
       <c r="J115" t="n">
-        <v>0.000131618556372004</v>
+        <v>0.00429356203148014</v>
       </c>
       <c r="K115" t="n">
-        <v>0.000332754077197683</v>
+        <v>0.0108573990967724</v>
       </c>
       <c r="L115" t="n">
-        <v>44</v>
+        <v>87</v>
       </c>
       <c r="M115" t="n">
-        <v>0.000474030661165038</v>
+        <v>0.0937287898212689</v>
       </c>
       <c r="N115" t="b">
         <v>0</v>
@@ -6089,25 +6089,25 @@
         <v>21</v>
       </c>
       <c r="G116" t="n">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="H116" t="n">
         <v>79711</v>
       </c>
       <c r="I116" t="n">
-        <v>0.000313632999209645</v>
+        <v>0.0176315166074886</v>
       </c>
       <c r="J116" t="n">
-        <v>0.000202976699230528</v>
+        <v>0.0127587794458442</v>
       </c>
       <c r="K116" t="n">
-        <v>0.000462949602102913</v>
+        <v>0.0237529031245067</v>
       </c>
       <c r="L116" t="n">
-        <v>76</v>
+        <v>149</v>
       </c>
       <c r="M116" t="n">
-        <v>0.00095344431759732</v>
+        <v>0.186925267528948</v>
       </c>
       <c r="N116" t="b">
         <v>0</v>
@@ -6142,22 +6142,22 @@
         <v>82162</v>
       </c>
       <c r="I117" t="n">
-        <v>0.000669409215939242</v>
+        <v>0.0178948454586211</v>
       </c>
       <c r="J117" t="n">
-        <v>0.000504329206431064</v>
+        <v>0.0134784650913666</v>
       </c>
       <c r="K117" t="n">
-        <v>0.000871240130576489</v>
+        <v>0.0232982489841465</v>
       </c>
       <c r="L117" t="n">
-        <v>42</v>
+        <v>77</v>
       </c>
       <c r="M117" t="n">
-        <v>0.000511185219444512</v>
+        <v>0.0937172902314939</v>
       </c>
       <c r="N117" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O117" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Regenerate ddPCR downstream outputs
</commit_message>
<xml_diff>
--- a/results/ddPCR/SNV_pooled_participant.xlsx
+++ b/results/ddPCR/SNV_pooled_participant.xlsx
@@ -778,25 +778,25 @@
         <v>21</v>
       </c>
       <c r="G3" t="n">
-        <v>115</v>
+        <v>67</v>
       </c>
       <c r="H3" t="n">
         <v>87610</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0253201539099395</v>
+        <v>0.0147492571433028</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0208902241817673</v>
+        <v>0.0114248255753369</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0304178244175161</v>
+        <v>0.0187430524364167</v>
       </c>
       <c r="L3" t="n">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="M3" t="n">
-        <v>0.151809154206141</v>
+        <v>0.106152265723091</v>
       </c>
       <c r="N3" t="b">
         <v>0</v>
@@ -919,25 +919,25 @@
         <v>21</v>
       </c>
       <c r="G6" t="n">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="H6" t="n">
         <v>83753</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0279045939839292</v>
+        <v>0.0224316521363432</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0227442223249464</v>
+        <v>0.0178345937108173</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0338902090542832</v>
+        <v>0.0278554745274867</v>
       </c>
       <c r="L6" t="n">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="M6" t="n">
-        <v>0.151636359294592</v>
+        <v>0.10745883729538</v>
       </c>
       <c r="N6" t="b">
         <v>0</v>
@@ -1060,19 +1060,19 @@
         <v>21</v>
       </c>
       <c r="G9" t="n">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="H9" t="n">
         <v>91460</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0269604404879219</v>
+        <v>0.024447205186745</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0229094737504563</v>
+        <v>0.0206023144232989</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0315340655634852</v>
+        <v>0.0288132392413934</v>
       </c>
       <c r="L9" t="n">
         <v>166</v>
@@ -1201,25 +1201,25 @@
         <v>21</v>
       </c>
       <c r="G12" t="n">
-        <v>106</v>
+        <v>65</v>
       </c>
       <c r="H12" t="n">
         <v>88866</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0333228963656859</v>
+        <v>0.020431768959649</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0272761607573691</v>
+        <v>0.0157662541403076</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0403139459986585</v>
+        <v>0.0260476125215893</v>
       </c>
       <c r="L12" t="n">
-        <v>135</v>
+        <v>95</v>
       </c>
       <c r="M12" t="n">
-        <v>0.151914117885355</v>
+        <v>0.106902527400806</v>
       </c>
       <c r="N12" t="b">
         <v>0</v>
@@ -1310,10 +1310,10 @@
         <v>0.0216468968986501</v>
       </c>
       <c r="L14" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M14" t="n">
-        <v>0.101424350663668</v>
+        <v>0.0984845144125472</v>
       </c>
       <c r="N14" t="b">
         <v>0</v>
@@ -1436,19 +1436,19 @@
         <v>20</v>
       </c>
       <c r="G17" t="n">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="H17" t="n">
         <v>84651</v>
       </c>
       <c r="I17" t="n">
-        <v>0.030283139964908</v>
+        <v>0.0190763440686068</v>
       </c>
       <c r="J17" t="n">
-        <v>0.0246328570103583</v>
+        <v>0.0146557466346035</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0368449595471133</v>
+        <v>0.0244137032657901</v>
       </c>
       <c r="L17" t="n">
         <v>200</v>
@@ -1483,19 +1483,19 @@
         <v>22</v>
       </c>
       <c r="G18" t="n">
-        <v>173</v>
+        <v>148</v>
       </c>
       <c r="H18" t="n">
         <v>90821</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0514092045052246</v>
+        <v>0.0439773368411513</v>
       </c>
       <c r="J18" t="n">
-        <v>0.044020382359506</v>
+        <v>0.0371673756035627</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0596879993344228</v>
+        <v>0.0516778462985493</v>
       </c>
       <c r="L18" t="n">
         <v>334</v>
@@ -1545,10 +1545,10 @@
         <v>0.0271423035055794</v>
       </c>
       <c r="L19" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="M19" t="n">
-        <v>0.101639430819187</v>
+        <v>0.0963594603870218</v>
       </c>
       <c r="N19" t="b">
         <v>0</v>
@@ -1718,25 +1718,25 @@
         <v>21</v>
       </c>
       <c r="G23" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="H23" t="n">
         <v>90154</v>
       </c>
       <c r="I23" t="n">
-        <v>0.0418049338415665</v>
+        <v>0.0331551938509705</v>
       </c>
       <c r="J23" t="n">
-        <v>0.0334817031091647</v>
+        <v>0.0257951617592695</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0515710491993853</v>
+        <v>0.0419635577172388</v>
       </c>
       <c r="L23" t="n">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="M23" t="n">
-        <v>0.171928034252501</v>
+        <v>0.157508263637775</v>
       </c>
       <c r="N23" t="b">
         <v>0</v>
@@ -1859,25 +1859,25 @@
         <v>21</v>
       </c>
       <c r="G26" t="n">
-        <v>489</v>
+        <v>404</v>
       </c>
       <c r="H26" t="n">
         <v>181499</v>
       </c>
       <c r="I26" t="n">
-        <v>0.125606358120142</v>
+        <v>0.103771277513502</v>
       </c>
       <c r="J26" t="n">
-        <v>0.114709868958417</v>
+        <v>0.0938912115561042</v>
       </c>
       <c r="K26" t="n">
-        <v>0.137260692967258</v>
+        <v>0.114409779360701</v>
       </c>
       <c r="L26" t="n">
-        <v>300</v>
+        <v>275</v>
       </c>
       <c r="M26" t="n">
-        <v>0.165290166887972</v>
+        <v>0.151515986313974</v>
       </c>
       <c r="N26" t="b">
         <v>1</v>
@@ -2000,25 +2000,25 @@
         <v>21</v>
       </c>
       <c r="G29" t="n">
-        <v>175</v>
+        <v>153</v>
       </c>
       <c r="H29" t="n">
         <v>94780</v>
       </c>
       <c r="I29" t="n">
-        <v>0.0397445286632307</v>
+        <v>0.0347457727016507</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0340552588161853</v>
+        <v>0.029443312212428</v>
       </c>
       <c r="K29" t="n">
-        <v>0.0461185365203327</v>
+        <v>0.040732768603473</v>
       </c>
       <c r="L29" t="n">
-        <v>162</v>
+        <v>84</v>
       </c>
       <c r="M29" t="n">
-        <v>0.170922135471618</v>
+        <v>0.0886262924667651</v>
       </c>
       <c r="N29" t="b">
         <v>1</v>
@@ -2047,19 +2047,19 @@
         <v>22</v>
       </c>
       <c r="G30" t="n">
-        <v>188</v>
+        <v>139</v>
       </c>
       <c r="H30" t="n">
         <v>89221</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0505261205414791</v>
+        <v>0.0373517286909395</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0435422136848823</v>
+        <v>0.0313888706567372</v>
       </c>
       <c r="K30" t="n">
-        <v>0.0583176125606386</v>
+        <v>0.0441224083906451</v>
       </c>
       <c r="L30" t="n">
         <v>328</v>
@@ -2094,19 +2094,19 @@
         <v>20</v>
       </c>
       <c r="G31" t="n">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="H31" t="n">
         <v>91262</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0231911357245898</v>
+        <v>0.00959584865470188</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0176085998339115</v>
+        <v>0.00614796790371202</v>
       </c>
       <c r="K31" t="n">
-        <v>0.029983258387406</v>
+        <v>0.0142789610986949</v>
       </c>
       <c r="L31" t="n">
         <v>139</v>
@@ -2141,19 +2141,19 @@
         <v>21</v>
       </c>
       <c r="G32" t="n">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="H32" t="n">
         <v>91832</v>
       </c>
       <c r="I32" t="n">
-        <v>0.0229563309349425</v>
+        <v>0.015429145722088</v>
       </c>
       <c r="J32" t="n">
-        <v>0.017558155595385</v>
+        <v>0.0110714265674864</v>
       </c>
       <c r="K32" t="n">
-        <v>0.0294921094759439</v>
+        <v>0.0209336175734054</v>
       </c>
       <c r="L32" t="n">
         <v>166</v>
@@ -2188,25 +2188,25 @@
         <v>22</v>
       </c>
       <c r="G33" t="n">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="H33" t="n">
         <v>85905</v>
       </c>
       <c r="I33" t="n">
-        <v>0.0361733552983198</v>
+        <v>0.0256880270870303</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0281434089962867</v>
+        <v>0.0190032678470916</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0457834108070701</v>
+        <v>0.0339633093424599</v>
       </c>
       <c r="L33" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="M33" t="n">
-        <v>0.186252255398405</v>
+        <v>0.139689191548804</v>
       </c>
       <c r="N33" t="b">
         <v>0</v>
@@ -2235,19 +2235,19 @@
         <v>20</v>
       </c>
       <c r="G34" t="n">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="H34" t="n">
         <v>91571</v>
       </c>
       <c r="I34" t="n">
-        <v>0.0170932050110588</v>
+        <v>0.0109876591873305</v>
       </c>
       <c r="J34" t="n">
-        <v>0.0133210112623035</v>
+        <v>0.00801264570307064</v>
       </c>
       <c r="K34" t="n">
-        <v>0.0216046657224494</v>
+        <v>0.0147070899130404</v>
       </c>
       <c r="L34" t="n">
         <v>139</v>
@@ -2282,19 +2282,19 @@
         <v>21</v>
       </c>
       <c r="G35" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="H35" t="n">
         <v>91934</v>
       </c>
       <c r="I35" t="n">
-        <v>0.0135531654762694</v>
+        <v>0.0109823625657922</v>
       </c>
       <c r="J35" t="n">
-        <v>0.0102883957633695</v>
+        <v>0.0080672972068428</v>
       </c>
       <c r="K35" t="n">
-        <v>0.0175276818894564</v>
+        <v>0.0146095977647829</v>
       </c>
       <c r="L35" t="n">
         <v>145</v>
@@ -2329,19 +2329,19 @@
         <v>22</v>
       </c>
       <c r="G36" t="n">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="H36" t="n">
         <v>99167</v>
       </c>
       <c r="I36" t="n">
-        <v>0.0210403743223182</v>
+        <v>0.0162673014848809</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0170559128515269</v>
+        <v>0.0127911283628353</v>
       </c>
       <c r="K36" t="n">
-        <v>0.0256794891378054</v>
+        <v>0.0203997151686332</v>
       </c>
       <c r="L36" t="n">
         <v>333</v>
@@ -2376,19 +2376,19 @@
         <v>20</v>
       </c>
       <c r="G37" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="H37" t="n">
         <v>132006</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0149545398999578</v>
+        <v>0.0112153467824458</v>
       </c>
       <c r="J37" t="n">
-        <v>0.0120521585822811</v>
+        <v>0.00872418669514652</v>
       </c>
       <c r="K37" t="n">
-        <v>0.0183467624469577</v>
+        <v>0.0141980614309609</v>
       </c>
       <c r="L37" t="n">
         <v>366</v>
@@ -2423,19 +2423,19 @@
         <v>21</v>
       </c>
       <c r="G38" t="n">
-        <v>116</v>
+        <v>76</v>
       </c>
       <c r="H38" t="n">
         <v>113540</v>
       </c>
       <c r="I38" t="n">
-        <v>0.0235355731401993</v>
+        <v>0.0154183921219199</v>
       </c>
       <c r="J38" t="n">
-        <v>0.0194421511101324</v>
+        <v>0.0121451322618665</v>
       </c>
       <c r="K38" t="n">
-        <v>0.0282389041012529</v>
+        <v>0.0193042001089457</v>
       </c>
       <c r="L38" t="n">
         <v>203</v>
@@ -2470,25 +2470,25 @@
         <v>22</v>
       </c>
       <c r="G39" t="n">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H39" t="n">
         <v>92874</v>
       </c>
       <c r="I39" t="n">
-        <v>0.0197262489321322</v>
+        <v>0.0126020142784466</v>
       </c>
       <c r="J39" t="n">
-        <v>0.0154313568195835</v>
+        <v>0.00922479442858349</v>
       </c>
       <c r="K39" t="n">
-        <v>0.0248487354700057</v>
+        <v>0.0168131021553524</v>
       </c>
       <c r="L39" t="n">
-        <v>172</v>
+        <v>95</v>
       </c>
       <c r="M39" t="n">
-        <v>0.18519714882529</v>
+        <v>0.102289122897689</v>
       </c>
       <c r="N39" t="b">
         <v>0</v>
@@ -2705,25 +2705,25 @@
         <v>21</v>
       </c>
       <c r="G44" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="H44" t="n">
         <v>74800</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0175611044917311</v>
+        <v>0.0102429254681825</v>
       </c>
       <c r="J44" t="n">
-        <v>0.0122986995679106</v>
+        <v>0.00634021873571245</v>
       </c>
       <c r="K44" t="n">
-        <v>0.0243146652263116</v>
+        <v>0.0156587944184686</v>
       </c>
       <c r="L44" t="n">
-        <v>130</v>
+        <v>67</v>
       </c>
       <c r="M44" t="n">
-        <v>0.17379679144385</v>
+        <v>0.089572192513369</v>
       </c>
       <c r="N44" t="b">
         <v>0</v>
@@ -2752,19 +2752,19 @@
         <v>22</v>
       </c>
       <c r="G45" t="n">
-        <v>165</v>
+        <v>139</v>
       </c>
       <c r="H45" t="n">
         <v>165442</v>
       </c>
       <c r="I45" t="n">
-        <v>0.0385047191563009</v>
+        <v>0.0324367270699377</v>
       </c>
       <c r="J45" t="n">
-        <v>0.0328512508921773</v>
+        <v>0.0272669187190761</v>
       </c>
       <c r="K45" t="n">
-        <v>0.0448527589403779</v>
+        <v>0.0383024065660537</v>
       </c>
       <c r="L45" t="n">
         <v>594</v>
@@ -2893,19 +2893,19 @@
         <v>22</v>
       </c>
       <c r="G48" t="n">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="H48" t="n">
         <v>86847</v>
       </c>
       <c r="I48" t="n">
-        <v>0.0230052754712556</v>
+        <v>0.0154839687461726</v>
       </c>
       <c r="J48" t="n">
-        <v>0.0171802453100389</v>
+        <v>0.0107845722005335</v>
       </c>
       <c r="K48" t="n">
-        <v>0.0301713774509772</v>
+        <v>0.0215362746033436</v>
       </c>
       <c r="L48" t="n">
         <v>116</v>
@@ -2940,25 +2940,25 @@
         <v>20</v>
       </c>
       <c r="G49" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H49" t="n">
         <v>78865</v>
       </c>
       <c r="I49" t="n">
-        <v>0.0147102222277732</v>
+        <v>0.0100297212703188</v>
       </c>
       <c r="J49" t="n">
-        <v>0.00921866570187686</v>
+        <v>0.00561349448655299</v>
       </c>
       <c r="K49" t="n">
-        <v>0.0222722808782927</v>
+        <v>0.0165430314451874</v>
       </c>
       <c r="L49" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="M49" t="n">
-        <v>0.106511126608762</v>
+        <v>0.0963672097888797</v>
       </c>
       <c r="N49" t="b">
         <v>0</v>
@@ -2987,19 +2987,19 @@
         <v>21</v>
       </c>
       <c r="G50" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="H50" t="n">
         <v>83855</v>
       </c>
       <c r="I50" t="n">
-        <v>0.0315981873500525</v>
+        <v>0.0248638939389279</v>
       </c>
       <c r="J50" t="n">
-        <v>0.0241686663711455</v>
+        <v>0.0183317356544619</v>
       </c>
       <c r="K50" t="n">
-        <v>0.0405926586045002</v>
+        <v>0.0329684537205359</v>
       </c>
       <c r="L50" t="n">
         <v>153</v>
@@ -3034,25 +3034,25 @@
         <v>22</v>
       </c>
       <c r="G51" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="H51" t="n">
         <v>82752</v>
       </c>
       <c r="I51" t="n">
-        <v>0.0272124650574152</v>
+        <v>0.0191820107841436</v>
       </c>
       <c r="J51" t="n">
-        <v>0.0208135404302072</v>
+        <v>0.01388113317232</v>
       </c>
       <c r="K51" t="n">
-        <v>0.0349598305068229</v>
+        <v>0.0258407646971285</v>
       </c>
       <c r="L51" t="n">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="M51" t="n">
-        <v>0.186098221191029</v>
+        <v>0.134135730858469</v>
       </c>
       <c r="N51" t="b">
         <v>0</v>
@@ -3175,19 +3175,19 @@
         <v>22</v>
       </c>
       <c r="G54" t="n">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="H54" t="n">
         <v>130652</v>
       </c>
       <c r="I54" t="n">
-        <v>0.0282064996113581</v>
+        <v>0.0226811185691278</v>
       </c>
       <c r="J54" t="n">
-        <v>0.0228719878845399</v>
+        <v>0.0179273943011885</v>
       </c>
       <c r="K54" t="n">
-        <v>0.0344126244765838</v>
+        <v>0.0283093664271166</v>
       </c>
       <c r="L54" t="n">
         <v>218</v>
@@ -3222,19 +3222,19 @@
         <v>20</v>
       </c>
       <c r="G55" t="n">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="H55" t="n">
         <v>107664</v>
       </c>
       <c r="I55" t="n">
-        <v>0.0182796023551768</v>
+        <v>0.0148867710608022</v>
       </c>
       <c r="J55" t="n">
-        <v>0.014817334169937</v>
+        <v>0.0117816306960839</v>
       </c>
       <c r="K55" t="n">
-        <v>0.0223111345908309</v>
+        <v>0.0185621414291045</v>
       </c>
       <c r="L55" t="n">
         <v>162</v>
@@ -3269,19 +3269,19 @@
         <v>21</v>
       </c>
       <c r="G56" t="n">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="H56" t="n">
         <v>104891</v>
       </c>
       <c r="I56" t="n">
-        <v>0.0244357388599961</v>
+        <v>0.0207699507944982</v>
       </c>
       <c r="J56" t="n">
-        <v>0.0193738404396642</v>
+        <v>0.016127032892081</v>
       </c>
       <c r="K56" t="n">
-        <v>0.030416875346045</v>
+        <v>0.0263344740602863</v>
       </c>
       <c r="L56" t="n">
         <v>189</v>
@@ -3316,19 +3316,19 @@
         <v>22</v>
       </c>
       <c r="G57" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="H57" t="n">
         <v>89610</v>
       </c>
       <c r="I57" t="n">
-        <v>0.0381540489179008</v>
+        <v>0.0352561139714008</v>
       </c>
       <c r="J57" t="n">
-        <v>0.0302049178138576</v>
+        <v>0.0276334215628157</v>
       </c>
       <c r="K57" t="n">
-        <v>0.0475556200361264</v>
+        <v>0.0443331331832153</v>
       </c>
       <c r="L57" t="n">
         <v>330</v>
@@ -3363,19 +3363,19 @@
         <v>20</v>
       </c>
       <c r="G58" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="H58" t="n">
         <v>93468</v>
       </c>
       <c r="I58" t="n">
-        <v>0.0135905120390037</v>
+        <v>0.00553637315589288</v>
       </c>
       <c r="J58" t="n">
-        <v>0.010207408756539</v>
+        <v>0.00346919754565199</v>
       </c>
       <c r="K58" t="n">
-        <v>0.0177379079046336</v>
+        <v>0.00838383981991075</v>
       </c>
       <c r="L58" t="n">
         <v>111</v>
@@ -3410,25 +3410,25 @@
         <v>21</v>
       </c>
       <c r="G59" t="n">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="H59" t="n">
         <v>97469</v>
       </c>
       <c r="I59" t="n">
-        <v>0.0120747618647055</v>
+        <v>0.00616547254221</v>
       </c>
       <c r="J59" t="n">
-        <v>0.0088706635948277</v>
+        <v>0.00394992704701602</v>
       </c>
       <c r="K59" t="n">
-        <v>0.0160604936853504</v>
+        <v>0.0091752992601241</v>
       </c>
       <c r="L59" t="n">
-        <v>135</v>
+        <v>79</v>
       </c>
       <c r="M59" t="n">
-        <v>0.138505576131898</v>
+        <v>0.0810514112179257</v>
       </c>
       <c r="N59" t="b">
         <v>0</v>
@@ -3457,25 +3457,25 @@
         <v>22</v>
       </c>
       <c r="G60" t="n">
-        <v>82</v>
+        <v>50</v>
       </c>
       <c r="H60" t="n">
         <v>86839</v>
       </c>
       <c r="I60" t="n">
-        <v>0.0249332915294612</v>
+        <v>0.0152019034270091</v>
       </c>
       <c r="J60" t="n">
-        <v>0.0198258421561042</v>
+        <v>0.0112813118444791</v>
       </c>
       <c r="K60" t="n">
-        <v>0.0309575154830267</v>
+        <v>0.0200463648388211</v>
       </c>
       <c r="L60" t="n">
-        <v>162</v>
+        <v>89</v>
       </c>
       <c r="M60" t="n">
-        <v>0.186552125197204</v>
+        <v>0.102488513225624</v>
       </c>
       <c r="N60" t="b">
         <v>0</v>
@@ -3504,19 +3504,19 @@
         <v>20</v>
       </c>
       <c r="G61" t="n">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="H61" t="n">
         <v>95425</v>
       </c>
       <c r="I61" t="n">
-        <v>0.0258513739132753</v>
+        <v>0.0202657394680822</v>
       </c>
       <c r="J61" t="n">
-        <v>0.021505529559729</v>
+        <v>0.0164441111084638</v>
       </c>
       <c r="K61" t="n">
-        <v>0.0308229213473843</v>
+        <v>0.0247133756953419</v>
       </c>
       <c r="L61" t="n">
         <v>269</v>
@@ -3551,19 +3551,19 @@
         <v>21</v>
       </c>
       <c r="G62" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="H62" t="n">
         <v>92988</v>
       </c>
       <c r="I62" t="n">
-        <v>0.0174286698746649</v>
+        <v>0.0124788617969452</v>
       </c>
       <c r="J62" t="n">
-        <v>0.0138345466175399</v>
+        <v>0.00947217201404054</v>
       </c>
       <c r="K62" t="n">
-        <v>0.0216748145327035</v>
+        <v>0.0161399038018023</v>
       </c>
       <c r="L62" t="n">
         <v>168</v>
@@ -3598,19 +3598,19 @@
         <v>22</v>
       </c>
       <c r="G63" t="n">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="H63" t="n">
         <v>119733</v>
       </c>
       <c r="I63" t="n">
-        <v>0.0214234935681378</v>
+        <v>0.0194753873835435</v>
       </c>
       <c r="J63" t="n">
-        <v>0.0177700859491449</v>
+        <v>0.0160008060310121</v>
       </c>
       <c r="K63" t="n">
-        <v>0.0256098167985612</v>
+        <v>0.023483186527801</v>
       </c>
       <c r="L63" t="n">
         <v>435</v>
@@ -3645,25 +3645,25 @@
         <v>20</v>
       </c>
       <c r="G64" t="n">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="H64" t="n">
         <v>78199</v>
       </c>
       <c r="I64" t="n">
-        <v>0.0409873116805308</v>
+        <v>0.0122099239207104</v>
       </c>
       <c r="J64" t="n">
-        <v>0.030115808540355</v>
+        <v>0.00667529608860902</v>
       </c>
       <c r="K64" t="n">
-        <v>0.0545054177265182</v>
+        <v>0.0204864094364336</v>
       </c>
       <c r="L64" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="M64" t="n">
-        <v>0.106139464699037</v>
+        <v>0.0971879435798412</v>
       </c>
       <c r="N64" t="b">
         <v>0</v>
@@ -3692,25 +3692,25 @@
         <v>21</v>
       </c>
       <c r="G65" t="n">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="H65" t="n">
         <v>76521</v>
       </c>
       <c r="I65" t="n">
-        <v>0.037473005012722</v>
+        <v>0.0189450852857021</v>
       </c>
       <c r="J65" t="n">
-        <v>0.030088999724761</v>
+        <v>0.0138171905722285</v>
       </c>
       <c r="K65" t="n">
-        <v>0.0461234073139839</v>
+        <v>0.0253539520169561</v>
       </c>
       <c r="L65" t="n">
-        <v>133</v>
+        <v>69</v>
       </c>
       <c r="M65" t="n">
-        <v>0.173808497013892</v>
+        <v>0.0901713255184851</v>
       </c>
       <c r="N65" t="b">
         <v>0</v>
@@ -3739,25 +3739,25 @@
         <v>22</v>
       </c>
       <c r="G66" t="n">
-        <v>146</v>
+        <v>113</v>
       </c>
       <c r="H66" t="n">
         <v>144433</v>
       </c>
       <c r="I66" t="n">
-        <v>0.0380563213307327</v>
+        <v>0.0294537173979836</v>
       </c>
       <c r="J66" t="n">
-        <v>0.0321311532690353</v>
+        <v>0.0242723362329736</v>
       </c>
       <c r="K66" t="n">
-        <v>0.0447586467653664</v>
+        <v>0.0354146305869525</v>
       </c>
       <c r="L66" t="n">
-        <v>261</v>
+        <v>240</v>
       </c>
       <c r="M66" t="n">
-        <v>0.180706625217229</v>
+        <v>0.166167011694003</v>
       </c>
       <c r="N66" t="b">
         <v>0</v>
@@ -3801,10 +3801,10 @@
         <v>0.0348794982986761</v>
       </c>
       <c r="L67" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="M67" t="n">
-        <v>0.102165623426146</v>
+        <v>0.0978487660982805</v>
       </c>
       <c r="N67" t="b">
         <v>0</v>
@@ -3848,10 +3848,10 @@
         <v>0.0251271488599988</v>
       </c>
       <c r="L68" t="n">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="M68" t="n">
-        <v>0.0938032973280273</v>
+        <v>0.0795906765207504</v>
       </c>
       <c r="N68" t="b">
         <v>0</v>
@@ -3942,10 +3942,10 @@
         <v>0.0281452580095622</v>
       </c>
       <c r="L70" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M70" t="n">
-        <v>0.100522452218769</v>
+        <v>0.0965544606838172</v>
       </c>
       <c r="N70" t="b">
         <v>0</v>
@@ -3989,10 +3989,10 @@
         <v>0.0313690927627339</v>
       </c>
       <c r="L71" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="M71" t="n">
-        <v>0.0927902013547369</v>
+        <v>0.0782088839989926</v>
       </c>
       <c r="N71" t="b">
         <v>0</v>
@@ -4130,10 +4130,10 @@
         <v>0.0335702507749955</v>
       </c>
       <c r="L74" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="M74" t="n">
-        <v>0.0926676705664311</v>
+        <v>0.0785101097854486</v>
       </c>
       <c r="N74" t="b">
         <v>0</v>
@@ -4162,19 +4162,19 @@
         <v>22</v>
       </c>
       <c r="G75" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="H75" t="n">
         <v>120845</v>
       </c>
       <c r="I75" t="n">
-        <v>0.0226971955687063</v>
+        <v>0.0200780663276206</v>
       </c>
       <c r="J75" t="n">
-        <v>0.0179397910617122</v>
+        <v>0.0156208020261706</v>
       </c>
       <c r="K75" t="n">
-        <v>0.0283300616822594</v>
+        <v>0.0254125713440654</v>
       </c>
       <c r="L75" t="n">
         <v>203</v>
@@ -4256,25 +4256,25 @@
         <v>21</v>
       </c>
       <c r="G77" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H77" t="n">
         <v>85848</v>
       </c>
       <c r="I77" t="n">
-        <v>0.0167428746951768</v>
+        <v>0.0160148536014634</v>
       </c>
       <c r="J77" t="n">
-        <v>0.0122566137427708</v>
+        <v>0.0116352404470373</v>
       </c>
       <c r="K77" t="n">
-        <v>0.0223359862769231</v>
+        <v>0.0215023462988666</v>
       </c>
       <c r="L77" t="n">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="M77" t="n">
-        <v>0.186375920231106</v>
+        <v>0.173562575715218</v>
       </c>
       <c r="N77" t="b">
         <v>0</v>
@@ -4303,19 +4303,19 @@
         <v>22</v>
       </c>
       <c r="G78" t="n">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="H78" t="n">
         <v>188739</v>
       </c>
       <c r="I78" t="n">
-        <v>0.0193175064415262</v>
+        <v>0.0165855756608195</v>
       </c>
       <c r="J78" t="n">
-        <v>0.0156995026381077</v>
+        <v>0.013247341990242</v>
       </c>
       <c r="K78" t="n">
-        <v>0.0235199454658413</v>
+        <v>0.0205096034508786</v>
       </c>
       <c r="L78" t="n">
         <v>310</v>
@@ -4365,10 +4365,10 @@
         <v>0.03412846818393</v>
       </c>
       <c r="L79" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="M79" t="n">
-        <v>0.101484378171387</v>
+        <v>0.0974250030445313</v>
       </c>
       <c r="N79" t="b">
         <v>0</v>
@@ -4412,10 +4412,10 @@
         <v>0.022883204343539</v>
       </c>
       <c r="L80" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="M80" t="n">
-        <v>0.0943067726771517</v>
+        <v>0.0797980384191283</v>
       </c>
       <c r="N80" t="b">
         <v>0</v>
@@ -4647,10 +4647,10 @@
         <v>0.110430069440483</v>
       </c>
       <c r="L85" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M85" t="n">
-        <v>0.126440011239112</v>
+        <v>0.119415566170273</v>
       </c>
       <c r="N85" t="b">
         <v>0</v>
@@ -4820,25 +4820,25 @@
         <v>21</v>
       </c>
       <c r="G89" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="H89" t="n">
         <v>92756</v>
       </c>
       <c r="I89" t="n">
-        <v>0.0388844257519165</v>
+        <v>0.0288040082077371</v>
       </c>
       <c r="J89" t="n">
-        <v>0.0292109931786612</v>
+        <v>0.0205779227413981</v>
       </c>
       <c r="K89" t="n">
-        <v>0.0507366742463916</v>
+        <v>0.039223520170591</v>
       </c>
       <c r="L89" t="n">
-        <v>159</v>
+        <v>120</v>
       </c>
       <c r="M89" t="n">
-        <v>0.171417482427013</v>
+        <v>0.129371684850576</v>
       </c>
       <c r="N89" t="b">
         <v>0</v>
@@ -5384,25 +5384,25 @@
         <v>21</v>
       </c>
       <c r="G101" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="H101" t="n">
         <v>72663</v>
       </c>
       <c r="I101" t="n">
-        <v>0.038720926552352</v>
+        <v>0.0248197725146963</v>
       </c>
       <c r="J101" t="n">
-        <v>0.0306035114703714</v>
+        <v>0.018419986594793</v>
       </c>
       <c r="K101" t="n">
-        <v>0.0483333530718642</v>
+        <v>0.0327261722221661</v>
       </c>
       <c r="L101" t="n">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="M101" t="n">
-        <v>0.188541623659909</v>
+        <v>0.176155677580061</v>
       </c>
       <c r="N101" t="b">
         <v>0</v>
@@ -5478,19 +5478,19 @@
         <v>20</v>
       </c>
       <c r="G103" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H103" t="n">
         <v>91644</v>
       </c>
       <c r="I103" t="n">
-        <v>0.0240268801302244</v>
+        <v>0.0195642300889421</v>
       </c>
       <c r="J103" t="n">
-        <v>0.0187278064169064</v>
+        <v>0.0148161333449524</v>
       </c>
       <c r="K103" t="n">
-        <v>0.0303615433460644</v>
+        <v>0.0253515650474506</v>
       </c>
       <c r="L103" t="n">
         <v>259</v>
@@ -5525,25 +5525,25 @@
         <v>21</v>
       </c>
       <c r="G104" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H104" t="n">
         <v>90133</v>
       </c>
       <c r="I104" t="n">
-        <v>0.0285339416540302</v>
+        <v>0.0229655826368835</v>
       </c>
       <c r="J104" t="n">
-        <v>0.0226907198958314</v>
+        <v>0.0177594010822476</v>
       </c>
       <c r="K104" t="n">
-        <v>0.0354245816921393</v>
+        <v>0.0292226759999898</v>
       </c>
       <c r="L104" t="n">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="M104" t="n">
-        <v>0.185281750302331</v>
+        <v>0.181953335626241</v>
       </c>
       <c r="N104" t="b">
         <v>0</v>
@@ -5666,25 +5666,25 @@
         <v>21</v>
       </c>
       <c r="G107" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H107" t="n">
         <v>90230</v>
       </c>
       <c r="I107" t="n">
-        <v>0.00530164679248969</v>
+        <v>0.00407817193460925</v>
       </c>
       <c r="J107" t="n">
-        <v>0.00282282503900076</v>
+        <v>0.0019555981277632</v>
       </c>
       <c r="K107" t="n">
-        <v>0.00906652577954669</v>
+        <v>0.00750031651404556</v>
       </c>
       <c r="L107" t="n">
-        <v>155</v>
+        <v>80</v>
       </c>
       <c r="M107" t="n">
-        <v>0.171783220658318</v>
+        <v>0.088662307436551</v>
       </c>
       <c r="N107" t="b">
         <v>0</v>
@@ -5807,25 +5807,25 @@
         <v>21</v>
       </c>
       <c r="G110" t="n">
-        <v>184</v>
+        <v>154</v>
       </c>
       <c r="H110" t="n">
         <v>175608</v>
       </c>
       <c r="I110" t="n">
-        <v>0.0488230042682513</v>
+        <v>0.0408624929807351</v>
       </c>
       <c r="J110" t="n">
-        <v>0.0420211737294389</v>
+        <v>0.0346621569761626</v>
       </c>
       <c r="K110" t="n">
-        <v>0.0564130506850896</v>
+        <v>0.0478525765877347</v>
       </c>
       <c r="L110" t="n">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="M110" t="n">
-        <v>0.165709990433238</v>
+        <v>0.151473736959592</v>
       </c>
       <c r="N110" t="b">
         <v>0</v>
@@ -5948,25 +5948,25 @@
         <v>21</v>
       </c>
       <c r="G113" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H113" t="n">
         <v>83186</v>
       </c>
       <c r="I113" t="n">
-        <v>0.024343356125354</v>
+        <v>0.0225400089292493</v>
       </c>
       <c r="J113" t="n">
-        <v>0.0182860407527915</v>
+        <v>0.0167283764550275</v>
       </c>
       <c r="K113" t="n">
-        <v>0.0317663496039385</v>
+        <v>0.0297194050469943</v>
       </c>
       <c r="L113" t="n">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="M113" t="n">
-        <v>0.186329430433006</v>
+        <v>0.174308176856683</v>
       </c>
       <c r="N113" t="b">
         <v>0</v>
@@ -6104,10 +6104,10 @@
         <v>0.0237529031245067</v>
       </c>
       <c r="L116" t="n">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="M116" t="n">
-        <v>0.186925267528948</v>
+        <v>0.174379947560563</v>
       </c>
       <c r="N116" t="b">
         <v>0</v>

</xml_diff>